<commit_message>
Güncel Fon ve Hisse Fiyatları
</commit_message>
<xml_diff>
--- a/piyasa_verileri.xlsx
+++ b/piyasa_verileri.xlsx
@@ -545,7 +545,7 @@
         </is>
       </c>
       <c r="H2" s="1" t="n">
-        <v>367.25</v>
+        <v>368.75</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -554,7 +554,7 @@
       </c>
       <c r="K2" s="1" t="inlineStr">
         <is>
-          <t>13.928,76</t>
+          <t>13.940,48</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="K3" s="1" t="inlineStr">
         <is>
-          <t>47,3600</t>
+          <t>47,3597</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
         </is>
       </c>
       <c r="H4" s="1" t="n">
-        <v>226.6</v>
+        <v>233</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -640,7 +640,7 @@
       </c>
       <c r="K4" s="1" t="inlineStr">
         <is>
-          <t>54,0097</t>
+          <t>54,0378</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
         </is>
       </c>
       <c r="H5" s="1" t="n">
-        <v>1986</v>
+        <v>2008</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -683,7 +683,7 @@
       </c>
       <c r="K5" s="1" t="inlineStr">
         <is>
-          <t>65,214</t>
+          <t>65,110</t>
         </is>
       </c>
     </row>
@@ -717,7 +717,7 @@
         </is>
       </c>
       <c r="H6" s="1" t="n">
-        <v>298.25</v>
+        <v>297</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -760,7 +760,7 @@
         </is>
       </c>
       <c r="H7" s="1" t="n">
-        <v>127.7</v>
+        <v>128.1</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -769,7 +769,7 @@
       </c>
       <c r="K7" s="1" t="inlineStr">
         <is>
-          <t>86,22</t>
+          <t>85,55</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
         </is>
       </c>
       <c r="H8" s="1" t="n">
-        <v>89.59999999999999</v>
+        <v>89.8</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -812,7 +812,7 @@
       </c>
       <c r="K8" s="1" t="inlineStr">
         <is>
-          <t>6.228,18</t>
+          <t>6.235,50</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
         </is>
       </c>
       <c r="H9" s="1" t="n">
-        <v>199.9</v>
+        <v>200.1</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -889,7 +889,7 @@
         </is>
       </c>
       <c r="H10" s="1" t="n">
-        <v>381.5</v>
+        <v>382</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -932,7 +932,7 @@
         </is>
       </c>
       <c r="H11" s="1" t="n">
-        <v>325.75</v>
+        <v>326.25</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
@@ -975,7 +975,7 @@
         </is>
       </c>
       <c r="H12" s="1" t="n">
-        <v>13.06</v>
+        <v>13.11</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
@@ -1061,7 +1061,7 @@
         </is>
       </c>
       <c r="H14" s="1" t="n">
-        <v>68.25</v>
+        <v>68.7</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
@@ -1070,7 +1070,7 @@
       </c>
       <c r="K14" s="1" t="inlineStr">
         <is>
-          <t>4.090,02</t>
+          <t>4.094,84</t>
         </is>
       </c>
     </row>
@@ -1104,7 +1104,7 @@
         </is>
       </c>
       <c r="H15" s="1" t="n">
-        <v>143</v>
+        <v>143.5</v>
       </c>
     </row>
     <row r="16">
@@ -1137,7 +1137,7 @@
         </is>
       </c>
       <c r="H16" s="1" t="n">
-        <v>30.52</v>
+        <v>30.66</v>
       </c>
     </row>
     <row r="17">
@@ -1170,7 +1170,7 @@
         </is>
       </c>
       <c r="H17" s="1" t="n">
-        <v>43.5</v>
+        <v>43.58</v>
       </c>
     </row>
     <row r="18">
@@ -1203,7 +1203,7 @@
         </is>
       </c>
       <c r="H18" s="1" t="n">
-        <v>298.25</v>
+        <v>298.5</v>
       </c>
     </row>
     <row r="19">
@@ -1236,7 +1236,7 @@
         </is>
       </c>
       <c r="H19" s="1" t="n">
-        <v>33.84</v>
+        <v>34.06</v>
       </c>
     </row>
     <row r="20">
@@ -1269,7 +1269,7 @@
         </is>
       </c>
       <c r="H20" s="1" t="n">
-        <v>78.7</v>
+        <v>79.05</v>
       </c>
     </row>
     <row r="21">
@@ -1302,7 +1302,7 @@
         </is>
       </c>
       <c r="H21" s="1" t="n">
-        <v>2625</v>
+        <v>2486</v>
       </c>
     </row>
     <row r="22">
@@ -1335,7 +1335,7 @@
         </is>
       </c>
       <c r="H22" s="1" t="n">
-        <v>36.26</v>
+        <v>36.38</v>
       </c>
     </row>
     <row r="23">
@@ -1368,7 +1368,7 @@
         </is>
       </c>
       <c r="H23" s="1" t="n">
-        <v>90.90000000000001</v>
+        <v>90.55</v>
       </c>
     </row>
     <row r="24">
@@ -1401,7 +1401,7 @@
         </is>
       </c>
       <c r="H24" s="1" t="n">
-        <v>104.2</v>
+        <v>104</v>
       </c>
     </row>
     <row r="25">
@@ -1434,7 +1434,7 @@
         </is>
       </c>
       <c r="H25" s="1" t="n">
-        <v>3362.5</v>
+        <v>3370</v>
       </c>
     </row>
     <row r="26">
@@ -1467,7 +1467,7 @@
         </is>
       </c>
       <c r="H26" s="1" t="n">
-        <v>54.15</v>
+        <v>54.1</v>
       </c>
     </row>
     <row r="27">
@@ -1500,7 +1500,7 @@
         </is>
       </c>
       <c r="H27" s="1" t="n">
-        <v>88.45</v>
+        <v>88.40000000000001</v>
       </c>
     </row>
     <row r="28">
@@ -1566,7 +1566,7 @@
         </is>
       </c>
       <c r="H29" s="1" t="n">
-        <v>49.8</v>
+        <v>49.7</v>
       </c>
     </row>
     <row r="30">
@@ -1599,7 +1599,7 @@
         </is>
       </c>
       <c r="H30" s="1" t="n">
-        <v>235.8</v>
+        <v>238.6</v>
       </c>
     </row>
     <row r="31">
@@ -1632,7 +1632,7 @@
         </is>
       </c>
       <c r="H31" s="1" t="n">
-        <v>425</v>
+        <v>425.75</v>
       </c>
     </row>
     <row r="32">
@@ -1698,7 +1698,7 @@
         </is>
       </c>
       <c r="H33" s="1" t="n">
-        <v>282</v>
+        <v>282.75</v>
       </c>
     </row>
     <row r="34">
@@ -1731,7 +1731,7 @@
         </is>
       </c>
       <c r="H34" s="1" t="n">
-        <v>6.58</v>
+        <v>6.59</v>
       </c>
     </row>
     <row r="35">
@@ -1764,7 +1764,7 @@
         </is>
       </c>
       <c r="H35" s="1" t="n">
-        <v>80.75</v>
+        <v>80.90000000000001</v>
       </c>
     </row>
     <row r="36">
@@ -1797,7 +1797,7 @@
         </is>
       </c>
       <c r="H36" s="1" t="n">
-        <v>105.5</v>
+        <v>104.5</v>
       </c>
     </row>
     <row r="37">
@@ -1830,7 +1830,7 @@
         </is>
       </c>
       <c r="H37" s="1" t="n">
-        <v>43.66</v>
+        <v>43.72</v>
       </c>
     </row>
     <row r="38">
@@ -1863,7 +1863,7 @@
         </is>
       </c>
       <c r="H38" s="1" t="n">
-        <v>676</v>
+        <v>670</v>
       </c>
     </row>
     <row r="39">
@@ -1896,7 +1896,7 @@
         </is>
       </c>
       <c r="H39" s="1" t="n">
-        <v>105.1</v>
+        <v>105.2</v>
       </c>
     </row>
     <row r="40">
@@ -1962,7 +1962,7 @@
         </is>
       </c>
       <c r="H41" s="1" t="n">
-        <v>11035</v>
+        <v>11052.5</v>
       </c>
     </row>
     <row r="42">
@@ -1995,7 +1995,7 @@
         </is>
       </c>
       <c r="H42" s="1" t="n">
-        <v>39.02</v>
+        <v>39.26</v>
       </c>
     </row>
     <row r="43">
@@ -2061,7 +2061,7 @@
         </is>
       </c>
       <c r="H44" s="1" t="n">
-        <v>164.3</v>
+        <v>164.7</v>
       </c>
     </row>
     <row r="45">
@@ -2127,7 +2127,7 @@
         </is>
       </c>
       <c r="H46" s="1" t="n">
-        <v>624.5</v>
+        <v>625</v>
       </c>
     </row>
     <row r="47">
@@ -2160,7 +2160,7 @@
         </is>
       </c>
       <c r="H47" s="1" t="n">
-        <v>21.18</v>
+        <v>21.1</v>
       </c>
     </row>
     <row r="48">
@@ -2226,7 +2226,7 @@
         </is>
       </c>
       <c r="H49" s="1" t="n">
-        <v>2625</v>
+        <v>2615</v>
       </c>
     </row>
     <row r="50">
@@ -2259,7 +2259,7 @@
         </is>
       </c>
       <c r="H50" s="1" t="n">
-        <v>95.34999999999999</v>
+        <v>95.15000000000001</v>
       </c>
     </row>
     <row r="51">
@@ -2292,7 +2292,7 @@
         </is>
       </c>
       <c r="H51" s="1" t="n">
-        <v>266.25</v>
+        <v>267.75</v>
       </c>
     </row>
     <row r="52">
@@ -2325,7 +2325,7 @@
         </is>
       </c>
       <c r="H52" s="1" t="n">
-        <v>35.72</v>
+        <v>35.76</v>
       </c>
     </row>
     <row r="53">
@@ -2358,7 +2358,7 @@
         </is>
       </c>
       <c r="H53" s="1" t="n">
-        <v>44.9</v>
+        <v>44.84</v>
       </c>
     </row>
     <row r="54">
@@ -2391,7 +2391,7 @@
         </is>
       </c>
       <c r="H54" s="1" t="n">
-        <v>18.14</v>
+        <v>18.13</v>
       </c>
     </row>
     <row r="55">
@@ -2424,7 +2424,7 @@
         </is>
       </c>
       <c r="H55" s="1" t="n">
-        <v>256.5</v>
+        <v>257</v>
       </c>
     </row>
     <row r="56">
@@ -2457,7 +2457,7 @@
         </is>
       </c>
       <c r="H56" s="1" t="n">
-        <v>9.609999999999999</v>
+        <v>9.67</v>
       </c>
     </row>
     <row r="57">
@@ -2490,7 +2490,7 @@
         </is>
       </c>
       <c r="H57" s="1" t="n">
-        <v>98.25</v>
+        <v>97.25</v>
       </c>
     </row>
     <row r="58">
@@ -2523,7 +2523,7 @@
         </is>
       </c>
       <c r="H58" s="1" t="n">
-        <v>34.6</v>
+        <v>34.4</v>
       </c>
     </row>
     <row r="59">
@@ -2589,7 +2589,7 @@
         </is>
       </c>
       <c r="H60" s="1" t="n">
-        <v>164.4</v>
+        <v>164.8</v>
       </c>
     </row>
     <row r="61">
@@ -2622,7 +2622,7 @@
         </is>
       </c>
       <c r="H61" s="1" t="n">
-        <v>163.5</v>
+        <v>163.3</v>
       </c>
     </row>
     <row r="62">
@@ -2688,7 +2688,7 @@
         </is>
       </c>
       <c r="H63" s="1" t="n">
-        <v>110.7</v>
+        <v>113.3</v>
       </c>
     </row>
     <row r="64">
@@ -2721,7 +2721,7 @@
         </is>
       </c>
       <c r="H64" s="1" t="n">
-        <v>397.25</v>
+        <v>399.5</v>
       </c>
     </row>
     <row r="65">
@@ -2774,7 +2774,7 @@
         </is>
       </c>
       <c r="D66" s="1" t="n">
-        <v>1.230394</v>
+        <v>1.226021</v>
       </c>
       <c r="F66" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
         </is>
       </c>
       <c r="H67" s="1" t="n">
-        <v>19.01</v>
+        <v>19.15</v>
       </c>
     </row>
     <row r="68">
@@ -2853,7 +2853,7 @@
         </is>
       </c>
       <c r="H68" s="1" t="n">
-        <v>6.04</v>
+        <v>6.05</v>
       </c>
     </row>
     <row r="69">
@@ -2886,7 +2886,7 @@
         </is>
       </c>
       <c r="H69" s="1" t="n">
-        <v>99.25</v>
+        <v>99.59999999999999</v>
       </c>
     </row>
     <row r="70">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="H70" s="1" t="n">
-        <v>202.3</v>
+        <v>203.4</v>
       </c>
     </row>
     <row r="71">
@@ -2952,7 +2952,7 @@
         </is>
       </c>
       <c r="H71" s="1" t="n">
-        <v>99.3</v>
+        <v>99.8</v>
       </c>
     </row>
     <row r="72">
@@ -2985,7 +2985,7 @@
         </is>
       </c>
       <c r="H72" s="1" t="n">
-        <v>183.7</v>
+        <v>183.6</v>
       </c>
     </row>
     <row r="73">
@@ -3018,7 +3018,7 @@
         </is>
       </c>
       <c r="H73" s="1" t="n">
-        <v>32.2</v>
+        <v>32.32</v>
       </c>
     </row>
     <row r="74">
@@ -3051,7 +3051,7 @@
         </is>
       </c>
       <c r="H74" s="1" t="n">
-        <v>232.8</v>
+        <v>234.1</v>
       </c>
     </row>
     <row r="75">
@@ -3117,7 +3117,7 @@
         </is>
       </c>
       <c r="H76" s="1" t="n">
-        <v>93.05</v>
+        <v>93.09999999999999</v>
       </c>
     </row>
     <row r="77">
@@ -3150,7 +3150,7 @@
         </is>
       </c>
       <c r="H77" s="1" t="n">
-        <v>42.4</v>
+        <v>42.5</v>
       </c>
     </row>
     <row r="78">
@@ -3183,7 +3183,7 @@
         </is>
       </c>
       <c r="H78" s="1" t="n">
-        <v>43.18</v>
+        <v>43.24</v>
       </c>
     </row>
     <row r="79">
@@ -3216,7 +3216,7 @@
         </is>
       </c>
       <c r="H79" s="1" t="n">
-        <v>135.6</v>
+        <v>134.6</v>
       </c>
     </row>
     <row r="80">
@@ -3249,7 +3249,7 @@
         </is>
       </c>
       <c r="H80" s="1" t="n">
-        <v>20.92</v>
+        <v>20.82</v>
       </c>
     </row>
     <row r="81">
@@ -3282,7 +3282,7 @@
         </is>
       </c>
       <c r="H81" s="1" t="n">
-        <v>34.48</v>
+        <v>34.42</v>
       </c>
     </row>
     <row r="82">
@@ -3348,7 +3348,7 @@
         </is>
       </c>
       <c r="H83" s="1" t="n">
-        <v>36.08</v>
+        <v>36.12</v>
       </c>
     </row>
     <row r="84">
@@ -3381,7 +3381,7 @@
         </is>
       </c>
       <c r="H84" s="1" t="n">
-        <v>1749</v>
+        <v>1745</v>
       </c>
     </row>
     <row r="85">
@@ -3414,7 +3414,7 @@
         </is>
       </c>
       <c r="H85" s="1" t="n">
-        <v>27.04</v>
+        <v>27.06</v>
       </c>
     </row>
     <row r="86">
@@ -3447,7 +3447,7 @@
         </is>
       </c>
       <c r="H86" s="1" t="n">
-        <v>206.1</v>
+        <v>205.9</v>
       </c>
     </row>
     <row r="87">
@@ -3480,7 +3480,7 @@
         </is>
       </c>
       <c r="H87" s="1" t="n">
-        <v>152.2</v>
+        <v>152.5</v>
       </c>
     </row>
     <row r="88">
@@ -3513,7 +3513,7 @@
         </is>
       </c>
       <c r="H88" s="1" t="n">
-        <v>38.08</v>
+        <v>37.72</v>
       </c>
     </row>
     <row r="89">
@@ -3546,7 +3546,7 @@
         </is>
       </c>
       <c r="H89" s="1" t="n">
-        <v>137.5</v>
+        <v>137.7</v>
       </c>
     </row>
     <row r="90">
@@ -3579,7 +3579,7 @@
         </is>
       </c>
       <c r="H90" s="1" t="n">
-        <v>162.8</v>
+        <v>162.7</v>
       </c>
     </row>
     <row r="91">
@@ -3612,7 +3612,7 @@
         </is>
       </c>
       <c r="H91" s="1" t="n">
-        <v>214.1</v>
+        <v>214.2</v>
       </c>
     </row>
     <row r="92">
@@ -3645,7 +3645,7 @@
         </is>
       </c>
       <c r="H92" s="1" t="n">
-        <v>1805</v>
+        <v>1807</v>
       </c>
     </row>
     <row r="93">
@@ -3711,7 +3711,7 @@
         </is>
       </c>
       <c r="H94" s="1" t="n">
-        <v>48.4</v>
+        <v>48.16</v>
       </c>
     </row>
     <row r="95">
@@ -3744,7 +3744,7 @@
         </is>
       </c>
       <c r="H95" s="1" t="n">
-        <v>12.4</v>
+        <v>12.51</v>
       </c>
     </row>
     <row r="96">
@@ -3777,7 +3777,7 @@
         </is>
       </c>
       <c r="H96" s="1" t="n">
-        <v>104.8</v>
+        <v>104.5</v>
       </c>
     </row>
     <row r="97">
@@ -3810,7 +3810,7 @@
         </is>
       </c>
       <c r="H97" s="1" t="n">
-        <v>238.5</v>
+        <v>238.1</v>
       </c>
     </row>
     <row r="98">
@@ -3843,7 +3843,7 @@
         </is>
       </c>
       <c r="H98" s="1" t="n">
-        <v>104.8</v>
+        <v>104.7</v>
       </c>
     </row>
     <row r="99">
@@ -3876,7 +3876,7 @@
         </is>
       </c>
       <c r="H99" s="1" t="n">
-        <v>401.75</v>
+        <v>404.75</v>
       </c>
     </row>
     <row r="100">
@@ -3909,7 +3909,7 @@
         </is>
       </c>
       <c r="H100" s="1" t="n">
-        <v>237.9</v>
+        <v>237.6</v>
       </c>
     </row>
     <row r="101">
@@ -3942,7 +3942,7 @@
         </is>
       </c>
       <c r="H101" s="1" t="n">
-        <v>17.26</v>
+        <v>17.42</v>
       </c>
     </row>
     <row r="102">
@@ -3975,7 +3975,7 @@
         </is>
       </c>
       <c r="H102" s="1" t="n">
-        <v>130.6</v>
+        <v>130.7</v>
       </c>
     </row>
     <row r="103">
@@ -4008,7 +4008,7 @@
         </is>
       </c>
       <c r="H103" s="1" t="n">
-        <v>9.31</v>
+        <v>9.27</v>
       </c>
     </row>
     <row r="104">
@@ -4041,7 +4041,7 @@
         </is>
       </c>
       <c r="H104" s="1" t="n">
-        <v>409.5</v>
+        <v>409</v>
       </c>
     </row>
     <row r="105">
@@ -4074,7 +4074,7 @@
         </is>
       </c>
       <c r="H105" s="1" t="n">
-        <v>37.6</v>
+        <v>37.68</v>
       </c>
     </row>
     <row r="106">
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="H106" s="1" t="n">
-        <v>18.72</v>
+        <v>18.8</v>
       </c>
     </row>
     <row r="107">
@@ -4140,7 +4140,7 @@
         </is>
       </c>
       <c r="H107" s="1" t="n">
-        <v>19.78</v>
+        <v>20.06</v>
       </c>
     </row>
     <row r="108">
@@ -4173,7 +4173,7 @@
         </is>
       </c>
       <c r="H108" s="1" t="n">
-        <v>328.25</v>
+        <v>328.5</v>
       </c>
     </row>
     <row r="109">
@@ -4206,7 +4206,7 @@
         </is>
       </c>
       <c r="H109" s="1" t="n">
-        <v>80.65000000000001</v>
+        <v>81.55</v>
       </c>
     </row>
     <row r="110">
@@ -4239,7 +4239,7 @@
         </is>
       </c>
       <c r="H110" s="1" t="n">
-        <v>20.96</v>
+        <v>20.98</v>
       </c>
     </row>
     <row r="111">
@@ -4272,7 +4272,7 @@
         </is>
       </c>
       <c r="H111" s="1" t="n">
-        <v>187.9</v>
+        <v>188</v>
       </c>
     </row>
     <row r="112">
@@ -4305,7 +4305,7 @@
         </is>
       </c>
       <c r="H112" s="1" t="n">
-        <v>1505</v>
+        <v>1503</v>
       </c>
     </row>
     <row r="113">
@@ -4338,7 +4338,7 @@
         </is>
       </c>
       <c r="H113" s="1" t="n">
-        <v>346.5</v>
+        <v>344.5</v>
       </c>
     </row>
     <row r="114">
@@ -4404,7 +4404,7 @@
         </is>
       </c>
       <c r="H115" s="1" t="n">
-        <v>106</v>
+        <v>106.9</v>
       </c>
     </row>
     <row r="116">
@@ -4437,7 +4437,7 @@
         </is>
       </c>
       <c r="H116" s="1" t="n">
-        <v>126.3</v>
+        <v>126.6</v>
       </c>
     </row>
     <row r="117">
@@ -4470,7 +4470,7 @@
         </is>
       </c>
       <c r="H117" s="1" t="n">
-        <v>91.75</v>
+        <v>92.09999999999999</v>
       </c>
     </row>
     <row r="118">
@@ -4503,7 +4503,7 @@
         </is>
       </c>
       <c r="H118" s="1" t="n">
-        <v>472.75</v>
+        <v>469</v>
       </c>
     </row>
     <row r="119">
@@ -4536,7 +4536,7 @@
         </is>
       </c>
       <c r="H119" s="1" t="n">
-        <v>16.67</v>
+        <v>16.73</v>
       </c>
     </row>
     <row r="120">
@@ -4602,7 +4602,7 @@
         </is>
       </c>
       <c r="H121" s="1" t="n">
-        <v>14.06</v>
+        <v>14.01</v>
       </c>
     </row>
     <row r="122">
@@ -4668,7 +4668,7 @@
         </is>
       </c>
       <c r="H123" s="1" t="n">
-        <v>26.4</v>
+        <v>26.26</v>
       </c>
     </row>
     <row r="124">
@@ -4701,7 +4701,7 @@
         </is>
       </c>
       <c r="H124" s="1" t="n">
-        <v>45.34</v>
+        <v>45.5</v>
       </c>
     </row>
     <row r="125">
@@ -4734,7 +4734,7 @@
         </is>
       </c>
       <c r="H125" s="1" t="n">
-        <v>52.8</v>
+        <v>52.75</v>
       </c>
     </row>
     <row r="126">
@@ -4767,7 +4767,7 @@
         </is>
       </c>
       <c r="H126" s="1" t="n">
-        <v>250.25</v>
+        <v>247.4</v>
       </c>
     </row>
     <row r="127">
@@ -4787,7 +4787,7 @@
         </is>
       </c>
       <c r="D127" s="1" t="n">
-        <v>2.901357</v>
+        <v>2.896772</v>
       </c>
       <c r="F127" t="inlineStr">
         <is>
@@ -4800,7 +4800,7 @@
         </is>
       </c>
       <c r="H127" s="1" t="n">
-        <v>42.32</v>
+        <v>42.28</v>
       </c>
     </row>
     <row r="128">
@@ -4833,7 +4833,7 @@
         </is>
       </c>
       <c r="H128" s="1" t="n">
-        <v>39.14</v>
+        <v>39.16</v>
       </c>
     </row>
     <row r="129">
@@ -4866,7 +4866,7 @@
         </is>
       </c>
       <c r="H129" s="1" t="n">
-        <v>116.5</v>
+        <v>116.6</v>
       </c>
     </row>
     <row r="130">
@@ -4965,7 +4965,7 @@
         </is>
       </c>
       <c r="H132" s="1" t="n">
-        <v>14.9</v>
+        <v>14.97</v>
       </c>
     </row>
     <row r="133">
@@ -4998,7 +4998,7 @@
         </is>
       </c>
       <c r="H133" s="1" t="n">
-        <v>52.2</v>
+        <v>52.1</v>
       </c>
     </row>
     <row r="134">
@@ -5064,7 +5064,7 @@
         </is>
       </c>
       <c r="H135" s="1" t="n">
-        <v>171.4</v>
+        <v>171.3</v>
       </c>
     </row>
     <row r="136">
@@ -5097,7 +5097,7 @@
         </is>
       </c>
       <c r="H136" s="1" t="n">
-        <v>68.3</v>
+        <v>67.84999999999999</v>
       </c>
     </row>
     <row r="137">
@@ -5130,7 +5130,7 @@
         </is>
       </c>
       <c r="H137" s="1" t="n">
-        <v>100.9</v>
+        <v>101.4</v>
       </c>
     </row>
     <row r="138">
@@ -5163,7 +5163,7 @@
         </is>
       </c>
       <c r="H138" s="1" t="n">
-        <v>25.76</v>
+        <v>25.86</v>
       </c>
     </row>
     <row r="139">
@@ -5196,7 +5196,7 @@
         </is>
       </c>
       <c r="H139" s="1" t="n">
-        <v>3.79</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="140">
@@ -5229,7 +5229,7 @@
         </is>
       </c>
       <c r="H140" s="1" t="n">
-        <v>13442.5</v>
+        <v>13485</v>
       </c>
     </row>
     <row r="141">
@@ -5295,7 +5295,7 @@
         </is>
       </c>
       <c r="H142" s="1" t="n">
-        <v>9.58</v>
+        <v>9.66</v>
       </c>
     </row>
     <row r="143">
@@ -5328,7 +5328,7 @@
         </is>
       </c>
       <c r="H143" s="1" t="n">
-        <v>2.96</v>
+        <v>2.97</v>
       </c>
     </row>
     <row r="144">
@@ -5394,7 +5394,7 @@
         </is>
       </c>
       <c r="H145" s="1" t="n">
-        <v>81.90000000000001</v>
+        <v>82.3</v>
       </c>
     </row>
     <row r="146">
@@ -5427,7 +5427,7 @@
         </is>
       </c>
       <c r="H146" s="1" t="n">
-        <v>10.05</v>
+        <v>10.03</v>
       </c>
     </row>
     <row r="147">
@@ -5460,7 +5460,7 @@
         </is>
       </c>
       <c r="H147" s="1" t="n">
-        <v>24.78</v>
+        <v>24.86</v>
       </c>
     </row>
     <row r="148">
@@ -5493,7 +5493,7 @@
         </is>
       </c>
       <c r="H148" s="1" t="n">
-        <v>43.94</v>
+        <v>40.66</v>
       </c>
     </row>
     <row r="149">
@@ -5526,7 +5526,7 @@
         </is>
       </c>
       <c r="H149" s="1" t="n">
-        <v>47.38</v>
+        <v>47.3</v>
       </c>
     </row>
     <row r="150">
@@ -5559,7 +5559,7 @@
         </is>
       </c>
       <c r="H150" s="1" t="n">
-        <v>140.1</v>
+        <v>141</v>
       </c>
     </row>
     <row r="151">
@@ -5592,7 +5592,7 @@
         </is>
       </c>
       <c r="H151" s="1" t="n">
-        <v>139.6</v>
+        <v>141.5</v>
       </c>
     </row>
     <row r="152">
@@ -5691,7 +5691,7 @@
         </is>
       </c>
       <c r="H154" s="1" t="n">
-        <v>71.34999999999999</v>
+        <v>70</v>
       </c>
     </row>
     <row r="155">
@@ -5757,7 +5757,7 @@
         </is>
       </c>
       <c r="H156" s="1" t="n">
-        <v>78.8</v>
+        <v>79.75</v>
       </c>
     </row>
     <row r="157">
@@ -5790,7 +5790,7 @@
         </is>
       </c>
       <c r="H157" s="1" t="n">
-        <v>43.74</v>
+        <v>43.8</v>
       </c>
     </row>
     <row r="158">
@@ -5823,7 +5823,7 @@
         </is>
       </c>
       <c r="H158" s="1" t="n">
-        <v>52.85</v>
+        <v>52.8</v>
       </c>
     </row>
     <row r="159">
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="H159" s="1" t="n">
-        <v>23.92</v>
+        <v>24.02</v>
       </c>
     </row>
     <row r="160">
@@ -5889,7 +5889,7 @@
         </is>
       </c>
       <c r="H160" s="1" t="n">
-        <v>159.1</v>
+        <v>158.3</v>
       </c>
     </row>
     <row r="161">
@@ -5922,7 +5922,7 @@
         </is>
       </c>
       <c r="H161" s="1" t="n">
-        <v>8.140000000000001</v>
+        <v>8.15</v>
       </c>
     </row>
     <row r="162">
@@ -5955,7 +5955,7 @@
         </is>
       </c>
       <c r="H162" s="1" t="n">
-        <v>42.02</v>
+        <v>42.18</v>
       </c>
     </row>
     <row r="163">
@@ -5988,7 +5988,7 @@
         </is>
       </c>
       <c r="H163" s="1" t="n">
-        <v>176.1</v>
+        <v>175.5</v>
       </c>
     </row>
     <row r="164">
@@ -6021,7 +6021,7 @@
         </is>
       </c>
       <c r="H164" s="1" t="n">
-        <v>35.5</v>
+        <v>35.8</v>
       </c>
     </row>
     <row r="165">
@@ -6087,7 +6087,7 @@
         </is>
       </c>
       <c r="H166" s="1" t="n">
-        <v>135.8</v>
+        <v>135.5</v>
       </c>
     </row>
     <row r="167">
@@ -6120,7 +6120,7 @@
         </is>
       </c>
       <c r="H167" s="1" t="n">
-        <v>1689</v>
+        <v>1710</v>
       </c>
     </row>
     <row r="168">
@@ -6153,7 +6153,7 @@
         </is>
       </c>
       <c r="H168" s="1" t="n">
-        <v>3850</v>
+        <v>3927.5</v>
       </c>
     </row>
     <row r="169">
@@ -6186,7 +6186,7 @@
         </is>
       </c>
       <c r="H169" s="1" t="n">
-        <v>12.14</v>
+        <v>12.16</v>
       </c>
     </row>
     <row r="170">
@@ -6219,7 +6219,7 @@
         </is>
       </c>
       <c r="H170" s="1" t="n">
-        <v>12.82</v>
+        <v>12.88</v>
       </c>
     </row>
     <row r="171">
@@ -6252,7 +6252,7 @@
         </is>
       </c>
       <c r="H171" s="1" t="n">
-        <v>4.87</v>
+        <v>4.88</v>
       </c>
     </row>
     <row r="172">
@@ -6285,7 +6285,7 @@
         </is>
       </c>
       <c r="H172" s="1" t="n">
-        <v>12.11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="173">
@@ -6318,7 +6318,7 @@
         </is>
       </c>
       <c r="H173" s="1" t="n">
-        <v>4817.5</v>
+        <v>4802.5</v>
       </c>
     </row>
     <row r="174">
@@ -6338,7 +6338,7 @@
         </is>
       </c>
       <c r="D174" s="1" t="n">
-        <v>4.163652</v>
+        <v>4.138717</v>
       </c>
       <c r="F174" t="inlineStr">
         <is>
@@ -6384,7 +6384,7 @@
         </is>
       </c>
       <c r="H175" s="1" t="n">
-        <v>25.1</v>
+        <v>25.12</v>
       </c>
     </row>
     <row r="176">
@@ -6417,7 +6417,7 @@
         </is>
       </c>
       <c r="H176" s="1" t="n">
-        <v>15.93</v>
+        <v>15.88</v>
       </c>
     </row>
     <row r="177">
@@ -6483,7 +6483,7 @@
         </is>
       </c>
       <c r="H178" s="1" t="n">
-        <v>5420</v>
+        <v>5455</v>
       </c>
     </row>
     <row r="179">
@@ -6516,7 +6516,7 @@
         </is>
       </c>
       <c r="H179" s="1" t="n">
-        <v>46.34</v>
+        <v>46.38</v>
       </c>
     </row>
     <row r="180">
@@ -6549,7 +6549,7 @@
         </is>
       </c>
       <c r="H180" s="1" t="n">
-        <v>16.12</v>
+        <v>16.14</v>
       </c>
     </row>
     <row r="181">
@@ -6582,7 +6582,7 @@
         </is>
       </c>
       <c r="H181" s="1" t="n">
-        <v>35.12</v>
+        <v>35.28</v>
       </c>
     </row>
     <row r="182">
@@ -6615,7 +6615,7 @@
         </is>
       </c>
       <c r="H182" s="1" t="n">
-        <v>51.9</v>
+        <v>51.85</v>
       </c>
     </row>
     <row r="183">
@@ -6648,7 +6648,7 @@
         </is>
       </c>
       <c r="H183" s="1" t="n">
-        <v>21.06</v>
+        <v>21.26</v>
       </c>
     </row>
     <row r="184">
@@ -6681,7 +6681,7 @@
         </is>
       </c>
       <c r="H184" s="1" t="n">
-        <v>12.27</v>
+        <v>12.23</v>
       </c>
     </row>
     <row r="185">
@@ -6714,7 +6714,7 @@
         </is>
       </c>
       <c r="H185" s="1" t="n">
-        <v>224.3</v>
+        <v>222.2</v>
       </c>
     </row>
     <row r="186">
@@ -6747,7 +6747,7 @@
         </is>
       </c>
       <c r="H186" s="1" t="n">
-        <v>26.12</v>
+        <v>26.08</v>
       </c>
     </row>
     <row r="187">
@@ -6780,7 +6780,7 @@
         </is>
       </c>
       <c r="H187" s="1" t="n">
-        <v>157</v>
+        <v>156.5</v>
       </c>
     </row>
     <row r="188">
@@ -6813,7 +6813,7 @@
         </is>
       </c>
       <c r="H188" s="1" t="n">
-        <v>127.3</v>
+        <v>127.6</v>
       </c>
     </row>
     <row r="189">
@@ -6846,7 +6846,7 @@
         </is>
       </c>
       <c r="H189" s="1" t="n">
-        <v>75.59999999999999</v>
+        <v>75.34999999999999</v>
       </c>
     </row>
     <row r="190">
@@ -6879,7 +6879,7 @@
         </is>
       </c>
       <c r="H190" s="1" t="n">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="191">
@@ -6912,7 +6912,7 @@
         </is>
       </c>
       <c r="H191" s="1" t="n">
-        <v>5.2</v>
+        <v>5.21</v>
       </c>
     </row>
     <row r="192">
@@ -6945,7 +6945,7 @@
         </is>
       </c>
       <c r="H192" s="1" t="n">
-        <v>14.45</v>
+        <v>14.5</v>
       </c>
     </row>
     <row r="193">
@@ -6978,7 +6978,7 @@
         </is>
       </c>
       <c r="H193" s="1" t="n">
-        <v>12.85</v>
+        <v>12.91</v>
       </c>
     </row>
     <row r="194">
@@ -7011,7 +7011,7 @@
         </is>
       </c>
       <c r="H194" s="1" t="n">
-        <v>9.83</v>
+        <v>9.81</v>
       </c>
     </row>
     <row r="195">
@@ -7044,7 +7044,7 @@
         </is>
       </c>
       <c r="H195" s="1" t="n">
-        <v>13.05</v>
+        <v>13.11</v>
       </c>
     </row>
     <row r="196">
@@ -7077,7 +7077,7 @@
         </is>
       </c>
       <c r="H196" s="1" t="n">
-        <v>20.04</v>
+        <v>20.1</v>
       </c>
     </row>
     <row r="197">
@@ -7110,7 +7110,7 @@
         </is>
       </c>
       <c r="H197" s="1" t="n">
-        <v>236</v>
+        <v>236.2</v>
       </c>
     </row>
     <row r="198">
@@ -7176,7 +7176,7 @@
         </is>
       </c>
       <c r="H199" s="1" t="n">
-        <v>20.26</v>
+        <v>20.22</v>
       </c>
     </row>
     <row r="200">
@@ -7209,7 +7209,7 @@
         </is>
       </c>
       <c r="H200" s="1" t="n">
-        <v>25.56</v>
+        <v>25.54</v>
       </c>
     </row>
     <row r="201">
@@ -7242,7 +7242,7 @@
         </is>
       </c>
       <c r="H201" s="1" t="n">
-        <v>45.62</v>
+        <v>46.7</v>
       </c>
     </row>
     <row r="202">
@@ -7308,7 +7308,7 @@
         </is>
       </c>
       <c r="H203" s="1" t="n">
-        <v>72.7</v>
+        <v>72.75</v>
       </c>
     </row>
     <row r="204">
@@ -7341,7 +7341,7 @@
         </is>
       </c>
       <c r="H204" s="1" t="n">
-        <v>61.75</v>
+        <v>62.1</v>
       </c>
     </row>
     <row r="205">
@@ -7374,7 +7374,7 @@
         </is>
       </c>
       <c r="H205" s="1" t="n">
-        <v>19.42</v>
+        <v>19.41</v>
       </c>
     </row>
     <row r="206">
@@ -7407,7 +7407,7 @@
         </is>
       </c>
       <c r="H206" s="1" t="n">
-        <v>35.54</v>
+        <v>35.3</v>
       </c>
     </row>
     <row r="207">
@@ -7440,7 +7440,7 @@
         </is>
       </c>
       <c r="H207" s="1" t="n">
-        <v>43.6</v>
+        <v>44.1</v>
       </c>
     </row>
     <row r="208">
@@ -7539,7 +7539,7 @@
         </is>
       </c>
       <c r="H210" s="1" t="n">
-        <v>44.9</v>
+        <v>45.18</v>
       </c>
     </row>
     <row r="211">
@@ -7572,7 +7572,7 @@
         </is>
       </c>
       <c r="H211" s="1" t="n">
-        <v>9.92</v>
+        <v>9.960000000000001</v>
       </c>
     </row>
     <row r="212">
@@ -7605,7 +7605,7 @@
         </is>
       </c>
       <c r="H212" s="1" t="n">
-        <v>3.35</v>
+        <v>3.37</v>
       </c>
     </row>
     <row r="213">
@@ -7671,7 +7671,7 @@
         </is>
       </c>
       <c r="H214" s="1" t="n">
-        <v>38.08</v>
+        <v>37.84</v>
       </c>
     </row>
     <row r="215">
@@ -7704,7 +7704,7 @@
         </is>
       </c>
       <c r="H215" s="1" t="n">
-        <v>133.4</v>
+        <v>133.1</v>
       </c>
     </row>
     <row r="216">
@@ -7737,7 +7737,7 @@
         </is>
       </c>
       <c r="H216" s="1" t="n">
-        <v>2.54</v>
+        <v>2.56</v>
       </c>
     </row>
     <row r="217">
@@ -7803,7 +7803,7 @@
         </is>
       </c>
       <c r="H218" s="1" t="n">
-        <v>502</v>
+        <v>505</v>
       </c>
     </row>
     <row r="219">
@@ -7869,7 +7869,7 @@
         </is>
       </c>
       <c r="H220" s="1" t="n">
-        <v>26.76</v>
+        <v>26.8</v>
       </c>
     </row>
     <row r="221">
@@ -7902,7 +7902,7 @@
         </is>
       </c>
       <c r="H221" s="1" t="n">
-        <v>15.14</v>
+        <v>15.12</v>
       </c>
     </row>
     <row r="222">
@@ -7935,7 +7935,7 @@
         </is>
       </c>
       <c r="H222" s="1" t="n">
-        <v>24.56</v>
+        <v>24.58</v>
       </c>
     </row>
     <row r="223">
@@ -7968,7 +7968,7 @@
         </is>
       </c>
       <c r="H223" s="1" t="n">
-        <v>4.07</v>
+        <v>4.06</v>
       </c>
     </row>
     <row r="224">
@@ -8001,7 +8001,7 @@
         </is>
       </c>
       <c r="H224" s="1" t="n">
-        <v>13.18</v>
+        <v>13.06</v>
       </c>
     </row>
     <row r="225">
@@ -8034,7 +8034,7 @@
         </is>
       </c>
       <c r="H225" s="1" t="n">
-        <v>8.630000000000001</v>
+        <v>8.720000000000001</v>
       </c>
     </row>
     <row r="226">
@@ -8067,7 +8067,7 @@
         </is>
       </c>
       <c r="H226" s="1" t="n">
-        <v>44.7</v>
+        <v>44.66</v>
       </c>
     </row>
     <row r="227">
@@ -8100,7 +8100,7 @@
         </is>
       </c>
       <c r="H227" s="1" t="n">
-        <v>4.56</v>
+        <v>4.54</v>
       </c>
     </row>
     <row r="228">
@@ -8133,7 +8133,7 @@
         </is>
       </c>
       <c r="H228" s="1" t="n">
-        <v>69.2</v>
+        <v>69.09999999999999</v>
       </c>
     </row>
     <row r="229">
@@ -8199,7 +8199,7 @@
         </is>
       </c>
       <c r="H230" s="1" t="n">
-        <v>10.53</v>
+        <v>10.51</v>
       </c>
     </row>
     <row r="231">
@@ -8232,7 +8232,7 @@
         </is>
       </c>
       <c r="H231" s="1" t="n">
-        <v>7.06</v>
+        <v>7.07</v>
       </c>
     </row>
     <row r="232">
@@ -8265,7 +8265,7 @@
         </is>
       </c>
       <c r="H232" s="1" t="n">
-        <v>64.09999999999999</v>
+        <v>64.45</v>
       </c>
     </row>
     <row r="233">
@@ -8298,7 +8298,7 @@
         </is>
       </c>
       <c r="H233" s="1" t="n">
-        <v>13.63</v>
+        <v>13.64</v>
       </c>
     </row>
     <row r="234">
@@ -8331,7 +8331,7 @@
         </is>
       </c>
       <c r="H234" s="1" t="n">
-        <v>70.05</v>
+        <v>70.34999999999999</v>
       </c>
     </row>
     <row r="235">
@@ -8364,7 +8364,7 @@
         </is>
       </c>
       <c r="H235" s="1" t="n">
-        <v>37.6</v>
+        <v>37.9</v>
       </c>
     </row>
     <row r="236">
@@ -8397,7 +8397,7 @@
         </is>
       </c>
       <c r="H236" s="1" t="n">
-        <v>36.9</v>
+        <v>36.88</v>
       </c>
     </row>
     <row r="237">
@@ -8463,7 +8463,7 @@
         </is>
       </c>
       <c r="H238" s="1" t="n">
-        <v>95.5</v>
+        <v>95.25</v>
       </c>
     </row>
     <row r="239">
@@ -8496,7 +8496,7 @@
         </is>
       </c>
       <c r="H239" s="1" t="n">
-        <v>40.64</v>
+        <v>40.5</v>
       </c>
     </row>
     <row r="240">
@@ -8529,7 +8529,7 @@
         </is>
       </c>
       <c r="H240" s="1" t="n">
-        <v>15.35</v>
+        <v>15.41</v>
       </c>
     </row>
     <row r="241">
@@ -8562,7 +8562,7 @@
         </is>
       </c>
       <c r="H241" s="1" t="n">
-        <v>501.5</v>
+        <v>500.5</v>
       </c>
     </row>
     <row r="242">
@@ -8628,7 +8628,7 @@
         </is>
       </c>
       <c r="H243" s="1" t="n">
-        <v>57.7</v>
+        <v>57.85</v>
       </c>
     </row>
     <row r="244">
@@ -8661,7 +8661,7 @@
         </is>
       </c>
       <c r="H244" s="1" t="n">
-        <v>20.84</v>
+        <v>20.9</v>
       </c>
     </row>
     <row r="245">
@@ -8694,7 +8694,7 @@
         </is>
       </c>
       <c r="H245" s="1" t="n">
-        <v>6.49</v>
+        <v>6.48</v>
       </c>
     </row>
     <row r="246">
@@ -8727,7 +8727,7 @@
         </is>
       </c>
       <c r="H246" s="1" t="n">
-        <v>41.68</v>
+        <v>41.14</v>
       </c>
     </row>
     <row r="247">
@@ -8793,7 +8793,7 @@
         </is>
       </c>
       <c r="H248" s="1" t="n">
-        <v>3.79</v>
+        <v>3.78</v>
       </c>
     </row>
     <row r="249">
@@ -8826,7 +8826,7 @@
         </is>
       </c>
       <c r="H249" s="1" t="n">
-        <v>30.4</v>
+        <v>30.44</v>
       </c>
     </row>
     <row r="250">
@@ -8859,7 +8859,7 @@
         </is>
       </c>
       <c r="H250" s="1" t="n">
-        <v>9.9</v>
+        <v>9.949999999999999</v>
       </c>
     </row>
     <row r="251">
@@ -8925,7 +8925,7 @@
         </is>
       </c>
       <c r="H252" s="1" t="n">
-        <v>25.32</v>
+        <v>25.44</v>
       </c>
     </row>
     <row r="253">
@@ -8958,7 +8958,7 @@
         </is>
       </c>
       <c r="H253" s="1" t="n">
-        <v>97.75</v>
+        <v>98.15000000000001</v>
       </c>
     </row>
     <row r="254">
@@ -8991,7 +8991,7 @@
         </is>
       </c>
       <c r="H254" s="1" t="n">
-        <v>291.5</v>
+        <v>290.25</v>
       </c>
     </row>
     <row r="255">
@@ -9024,7 +9024,7 @@
         </is>
       </c>
       <c r="H255" s="1" t="n">
-        <v>10.78</v>
+        <v>10.74</v>
       </c>
     </row>
     <row r="256">
@@ -9057,7 +9057,7 @@
         </is>
       </c>
       <c r="H256" s="1" t="n">
-        <v>6.1</v>
+        <v>6.11</v>
       </c>
     </row>
     <row r="257">
@@ -9090,7 +9090,7 @@
         </is>
       </c>
       <c r="H257" s="1" t="n">
-        <v>34.9</v>
+        <v>34.76</v>
       </c>
     </row>
     <row r="258">
@@ -9123,7 +9123,7 @@
         </is>
       </c>
       <c r="H258" s="1" t="n">
-        <v>82.09999999999999</v>
+        <v>82.05</v>
       </c>
     </row>
     <row r="259">
@@ -9156,7 +9156,7 @@
         </is>
       </c>
       <c r="H259" s="1" t="n">
-        <v>80.75</v>
+        <v>80.90000000000001</v>
       </c>
     </row>
     <row r="260">
@@ -9222,7 +9222,7 @@
         </is>
       </c>
       <c r="H261" s="1" t="n">
-        <v>390.75</v>
+        <v>391.25</v>
       </c>
     </row>
     <row r="262">
@@ -9255,7 +9255,7 @@
         </is>
       </c>
       <c r="H262" s="1" t="n">
-        <v>18.16</v>
+        <v>18.23</v>
       </c>
     </row>
     <row r="263">
@@ -9288,7 +9288,7 @@
         </is>
       </c>
       <c r="H263" s="1" t="n">
-        <v>54.1</v>
+        <v>53.8</v>
       </c>
     </row>
     <row r="264">
@@ -9321,7 +9321,7 @@
         </is>
       </c>
       <c r="H264" s="1" t="n">
-        <v>123.5</v>
+        <v>123.6</v>
       </c>
     </row>
     <row r="265">
@@ -9354,7 +9354,7 @@
         </is>
       </c>
       <c r="H265" s="1" t="n">
-        <v>821.5</v>
+        <v>822.5</v>
       </c>
     </row>
     <row r="266">
@@ -9387,7 +9387,7 @@
         </is>
       </c>
       <c r="H266" s="1" t="n">
-        <v>2.64</v>
+        <v>2.65</v>
       </c>
     </row>
     <row r="267">
@@ -9420,7 +9420,7 @@
         </is>
       </c>
       <c r="H267" s="1" t="n">
-        <v>23.3</v>
+        <v>23.64</v>
       </c>
     </row>
     <row r="268">
@@ -9453,7 +9453,7 @@
         </is>
       </c>
       <c r="H268" s="1" t="n">
-        <v>241.4</v>
+        <v>242.1</v>
       </c>
     </row>
     <row r="269">
@@ -9486,7 +9486,7 @@
         </is>
       </c>
       <c r="H269" s="1" t="n">
-        <v>1072</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="270">
@@ -9519,7 +9519,7 @@
         </is>
       </c>
       <c r="H270" s="1" t="n">
-        <v>49.22</v>
+        <v>49.24</v>
       </c>
     </row>
     <row r="271">
@@ -9585,7 +9585,7 @@
         </is>
       </c>
       <c r="H272" s="1" t="n">
-        <v>6.99</v>
+        <v>6.98</v>
       </c>
     </row>
     <row r="273">
@@ -9618,7 +9618,7 @@
         </is>
       </c>
       <c r="H273" s="1" t="n">
-        <v>13.67</v>
+        <v>13.69</v>
       </c>
     </row>
     <row r="274">
@@ -9651,7 +9651,7 @@
         </is>
       </c>
       <c r="H274" s="1" t="n">
-        <v>22.94</v>
+        <v>22.92</v>
       </c>
     </row>
     <row r="275">
@@ -9684,7 +9684,7 @@
         </is>
       </c>
       <c r="H275" s="1" t="n">
-        <v>2.19</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="276">
@@ -9717,7 +9717,7 @@
         </is>
       </c>
       <c r="H276" s="1" t="n">
-        <v>17.43</v>
+        <v>17.39</v>
       </c>
     </row>
     <row r="277">
@@ -9750,7 +9750,7 @@
         </is>
       </c>
       <c r="H277" s="1" t="n">
-        <v>13.59</v>
+        <v>13.57</v>
       </c>
     </row>
     <row r="278">
@@ -9783,7 +9783,7 @@
         </is>
       </c>
       <c r="H278" s="1" t="n">
-        <v>31.66</v>
+        <v>31.58</v>
       </c>
     </row>
     <row r="279">
@@ -9849,7 +9849,7 @@
         </is>
       </c>
       <c r="H280" s="1" t="n">
-        <v>7.74</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="281">
@@ -9882,7 +9882,7 @@
         </is>
       </c>
       <c r="H281" s="1" t="n">
-        <v>113.6</v>
+        <v>112.6</v>
       </c>
     </row>
     <row r="282">
@@ -9915,7 +9915,7 @@
         </is>
       </c>
       <c r="H282" s="1" t="n">
-        <v>63.8</v>
+        <v>64</v>
       </c>
     </row>
     <row r="283">
@@ -9948,7 +9948,7 @@
         </is>
       </c>
       <c r="H283" s="1" t="n">
-        <v>420.25</v>
+        <v>420.5</v>
       </c>
     </row>
     <row r="284">
@@ -10014,7 +10014,7 @@
         </is>
       </c>
       <c r="H285" s="1" t="n">
-        <v>16.86</v>
+        <v>17.18</v>
       </c>
     </row>
     <row r="286">
@@ -10047,7 +10047,7 @@
         </is>
       </c>
       <c r="H286" s="1" t="n">
-        <v>11.17</v>
+        <v>11.19</v>
       </c>
     </row>
     <row r="287">
@@ -10080,7 +10080,7 @@
         </is>
       </c>
       <c r="H287" s="1" t="n">
-        <v>2.01</v>
+        <v>2</v>
       </c>
     </row>
     <row r="288">
@@ -10113,7 +10113,7 @@
         </is>
       </c>
       <c r="H288" s="1" t="n">
-        <v>23.86</v>
+        <v>23.98</v>
       </c>
     </row>
     <row r="289">
@@ -10179,7 +10179,7 @@
         </is>
       </c>
       <c r="H290" s="1" t="n">
-        <v>21.94</v>
+        <v>21.9</v>
       </c>
     </row>
     <row r="291">
@@ -10212,7 +10212,7 @@
         </is>
       </c>
       <c r="H291" s="1" t="n">
-        <v>10.07</v>
+        <v>10.1</v>
       </c>
     </row>
     <row r="292">
@@ -10245,7 +10245,7 @@
         </is>
       </c>
       <c r="H292" s="1" t="n">
-        <v>37.74</v>
+        <v>37.86</v>
       </c>
     </row>
     <row r="293">
@@ -10278,7 +10278,7 @@
         </is>
       </c>
       <c r="H293" s="1" t="n">
-        <v>6.18</v>
+        <v>6.16</v>
       </c>
     </row>
     <row r="294">
@@ -10311,7 +10311,7 @@
         </is>
       </c>
       <c r="H294" s="1" t="n">
-        <v>5.27</v>
+        <v>5.28</v>
       </c>
     </row>
     <row r="295">
@@ -10344,7 +10344,7 @@
         </is>
       </c>
       <c r="H295" s="1" t="n">
-        <v>29.9</v>
+        <v>29.96</v>
       </c>
     </row>
     <row r="296">
@@ -10377,7 +10377,7 @@
         </is>
       </c>
       <c r="H296" s="1" t="n">
-        <v>11.2</v>
+        <v>11.18</v>
       </c>
     </row>
     <row r="297">
@@ -10476,7 +10476,7 @@
         </is>
       </c>
       <c r="H299" s="1" t="n">
-        <v>10.48</v>
+        <v>10.51</v>
       </c>
     </row>
     <row r="300">
@@ -10509,7 +10509,7 @@
         </is>
       </c>
       <c r="H300" s="1" t="n">
-        <v>7.54</v>
+        <v>7.55</v>
       </c>
     </row>
     <row r="301">
@@ -10542,7 +10542,7 @@
         </is>
       </c>
       <c r="H301" s="1" t="n">
-        <v>11.61</v>
+        <v>11.63</v>
       </c>
     </row>
     <row r="302">
@@ -10575,7 +10575,7 @@
         </is>
       </c>
       <c r="H302" s="1" t="n">
-        <v>36.14</v>
+        <v>36.96</v>
       </c>
     </row>
     <row r="303">
@@ -10608,7 +10608,7 @@
         </is>
       </c>
       <c r="H303" s="1" t="n">
-        <v>45.7</v>
+        <v>45.86</v>
       </c>
     </row>
     <row r="304">
@@ -10641,7 +10641,7 @@
         </is>
       </c>
       <c r="H304" s="1" t="n">
-        <v>18.2</v>
+        <v>18.11</v>
       </c>
     </row>
     <row r="305">
@@ -10674,7 +10674,7 @@
         </is>
       </c>
       <c r="H305" s="1" t="n">
-        <v>12.26</v>
+        <v>12.24</v>
       </c>
     </row>
     <row r="306">
@@ -10740,7 +10740,7 @@
         </is>
       </c>
       <c r="H307" s="1" t="n">
-        <v>11.99</v>
+        <v>12.01</v>
       </c>
     </row>
     <row r="308">
@@ -10773,7 +10773,7 @@
         </is>
       </c>
       <c r="H308" s="1" t="n">
-        <v>22.58</v>
+        <v>22.52</v>
       </c>
     </row>
     <row r="309">
@@ -10839,7 +10839,7 @@
         </is>
       </c>
       <c r="H310" s="1" t="n">
-        <v>51.05</v>
+        <v>51.1</v>
       </c>
     </row>
     <row r="311">
@@ -10872,7 +10872,7 @@
         </is>
       </c>
       <c r="H311" s="1" t="n">
-        <v>16.54</v>
+        <v>16.55</v>
       </c>
     </row>
     <row r="312">
@@ -10905,7 +10905,7 @@
         </is>
       </c>
       <c r="H312" s="1" t="n">
-        <v>0.96</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="313">
@@ -10938,7 +10938,7 @@
         </is>
       </c>
       <c r="H313" s="1" t="n">
-        <v>18.75</v>
+        <v>18.79</v>
       </c>
     </row>
     <row r="314">
@@ -10971,7 +10971,7 @@
         </is>
       </c>
       <c r="H314" s="1" t="n">
-        <v>42.7</v>
+        <v>42.46</v>
       </c>
     </row>
     <row r="315">
@@ -11004,7 +11004,7 @@
         </is>
       </c>
       <c r="H315" s="1" t="n">
-        <v>106.6</v>
+        <v>106.1</v>
       </c>
     </row>
     <row r="316">
@@ -11037,7 +11037,7 @@
         </is>
       </c>
       <c r="H316" s="1" t="n">
-        <v>3.49</v>
+        <v>3.51</v>
       </c>
     </row>
     <row r="317">
@@ -11070,7 +11070,7 @@
         </is>
       </c>
       <c r="H317" s="1" t="n">
-        <v>9.039999999999999</v>
+        <v>9.050000000000001</v>
       </c>
     </row>
     <row r="318">
@@ -11103,7 +11103,7 @@
         </is>
       </c>
       <c r="H318" s="1" t="n">
-        <v>80.05</v>
+        <v>80.2</v>
       </c>
     </row>
     <row r="319">
@@ -11136,7 +11136,7 @@
         </is>
       </c>
       <c r="H319" s="1" t="n">
-        <v>13.68</v>
+        <v>13.69</v>
       </c>
     </row>
     <row r="320">
@@ -11169,7 +11169,7 @@
         </is>
       </c>
       <c r="H320" s="1" t="n">
-        <v>5.96</v>
+        <v>5.94</v>
       </c>
     </row>
     <row r="321">
@@ -11202,7 +11202,7 @@
         </is>
       </c>
       <c r="H321" s="1" t="n">
-        <v>173.8</v>
+        <v>174.6</v>
       </c>
     </row>
     <row r="322">
@@ -11235,7 +11235,7 @@
         </is>
       </c>
       <c r="H322" s="1" t="n">
-        <v>250.25</v>
+        <v>246.7</v>
       </c>
     </row>
     <row r="323">
@@ -11268,7 +11268,7 @@
         </is>
       </c>
       <c r="H323" s="1" t="n">
-        <v>2.21</v>
+        <v>2.22</v>
       </c>
     </row>
     <row r="324">
@@ -11301,7 +11301,7 @@
         </is>
       </c>
       <c r="H324" s="1" t="n">
-        <v>8.99</v>
+        <v>8.91</v>
       </c>
     </row>
     <row r="325">
@@ -11367,7 +11367,7 @@
         </is>
       </c>
       <c r="H326" s="1" t="n">
-        <v>16.94</v>
+        <v>16.87</v>
       </c>
     </row>
     <row r="327">
@@ -11400,7 +11400,7 @@
         </is>
       </c>
       <c r="H327" s="1" t="n">
-        <v>117.1</v>
+        <v>117.5</v>
       </c>
     </row>
     <row r="328">
@@ -11433,7 +11433,7 @@
         </is>
       </c>
       <c r="H328" s="1" t="n">
-        <v>32.04</v>
+        <v>32</v>
       </c>
     </row>
     <row r="329">
@@ -11466,7 +11466,7 @@
         </is>
       </c>
       <c r="H329" s="1" t="n">
-        <v>21.54</v>
+        <v>21.56</v>
       </c>
     </row>
     <row r="330">
@@ -11532,7 +11532,7 @@
         </is>
       </c>
       <c r="H331" s="1" t="n">
-        <v>4.69</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="332">
@@ -11565,7 +11565,7 @@
         </is>
       </c>
       <c r="H332" s="1" t="n">
-        <v>3.72</v>
+        <v>3.73</v>
       </c>
     </row>
     <row r="333">
@@ -11598,7 +11598,7 @@
         </is>
       </c>
       <c r="H333" s="1" t="n">
-        <v>6.71</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="334">
@@ -11631,7 +11631,7 @@
         </is>
       </c>
       <c r="H334" s="1" t="n">
-        <v>10.39</v>
+        <v>10.38</v>
       </c>
     </row>
     <row r="335">
@@ -11664,7 +11664,7 @@
         </is>
       </c>
       <c r="H335" s="1" t="n">
-        <v>27.6</v>
+        <v>27.76</v>
       </c>
     </row>
     <row r="336">
@@ -11697,7 +11697,7 @@
         </is>
       </c>
       <c r="H336" s="1" t="n">
-        <v>9.369999999999999</v>
+        <v>9.359999999999999</v>
       </c>
     </row>
     <row r="337">
@@ -11730,7 +11730,7 @@
         </is>
       </c>
       <c r="H337" s="1" t="n">
-        <v>6.26</v>
+        <v>6.27</v>
       </c>
     </row>
     <row r="338">
@@ -11763,7 +11763,7 @@
         </is>
       </c>
       <c r="H338" s="1" t="n">
-        <v>3.52</v>
+        <v>3.51</v>
       </c>
     </row>
     <row r="339">
@@ -11796,7 +11796,7 @@
         </is>
       </c>
       <c r="H339" s="1" t="n">
-        <v>31.3</v>
+        <v>31.38</v>
       </c>
     </row>
     <row r="340">
@@ -11829,7 +11829,7 @@
         </is>
       </c>
       <c r="H340" s="1" t="n">
-        <v>6.23</v>
+        <v>6.24</v>
       </c>
     </row>
     <row r="341">
@@ -11862,7 +11862,7 @@
         </is>
       </c>
       <c r="H341" s="1" t="n">
-        <v>434</v>
+        <v>438</v>
       </c>
     </row>
     <row r="342">
@@ -11895,7 +11895,7 @@
         </is>
       </c>
       <c r="H342" s="1" t="n">
-        <v>253.75</v>
+        <v>254</v>
       </c>
     </row>
     <row r="343">
@@ -11928,7 +11928,7 @@
         </is>
       </c>
       <c r="H343" s="1" t="n">
-        <v>858</v>
+        <v>849</v>
       </c>
     </row>
     <row r="344">
@@ -11961,7 +11961,7 @@
         </is>
       </c>
       <c r="H344" s="1" t="n">
-        <v>13.77</v>
+        <v>13.72</v>
       </c>
     </row>
     <row r="345">
@@ -12027,7 +12027,7 @@
         </is>
       </c>
       <c r="H346" s="1" t="n">
-        <v>2.58</v>
+        <v>2.59</v>
       </c>
     </row>
     <row r="347">
@@ -12060,7 +12060,7 @@
         </is>
       </c>
       <c r="H347" s="1" t="n">
-        <v>30.58</v>
+        <v>30.68</v>
       </c>
     </row>
     <row r="348">
@@ -12093,7 +12093,7 @@
         </is>
       </c>
       <c r="H348" s="1" t="n">
-        <v>71.90000000000001</v>
+        <v>72.5</v>
       </c>
     </row>
     <row r="349">
@@ -12126,7 +12126,7 @@
         </is>
       </c>
       <c r="H349" s="1" t="n">
-        <v>13.11</v>
+        <v>13.08</v>
       </c>
     </row>
     <row r="350">
@@ -12225,7 +12225,7 @@
         </is>
       </c>
       <c r="H352" s="1" t="n">
-        <v>31.78</v>
+        <v>31.72</v>
       </c>
     </row>
     <row r="353">
@@ -12258,7 +12258,7 @@
         </is>
       </c>
       <c r="H353" s="1" t="n">
-        <v>16.78</v>
+        <v>16.75</v>
       </c>
     </row>
     <row r="354">
@@ -12291,7 +12291,7 @@
         </is>
       </c>
       <c r="H354" s="1" t="n">
-        <v>22.18</v>
+        <v>22.16</v>
       </c>
     </row>
     <row r="355">
@@ -12324,7 +12324,7 @@
         </is>
       </c>
       <c r="H355" s="1" t="n">
-        <v>59.3</v>
+        <v>59.25</v>
       </c>
     </row>
     <row r="356">
@@ -12357,7 +12357,7 @@
         </is>
       </c>
       <c r="H356" s="1" t="n">
-        <v>33.9</v>
+        <v>33.92</v>
       </c>
     </row>
     <row r="357">
@@ -12390,7 +12390,7 @@
         </is>
       </c>
       <c r="H357" s="1" t="n">
-        <v>13.62</v>
+        <v>13.66</v>
       </c>
     </row>
     <row r="358">
@@ -12423,7 +12423,7 @@
         </is>
       </c>
       <c r="H358" s="1" t="n">
-        <v>6.51</v>
+        <v>6.53</v>
       </c>
     </row>
     <row r="359">
@@ -12489,7 +12489,7 @@
         </is>
       </c>
       <c r="H360" s="1" t="n">
-        <v>137.5</v>
+        <v>137.1</v>
       </c>
     </row>
     <row r="361">
@@ -12522,7 +12522,7 @@
         </is>
       </c>
       <c r="H361" s="1" t="n">
-        <v>13.12</v>
+        <v>13.16</v>
       </c>
     </row>
     <row r="362">
@@ -12555,7 +12555,7 @@
         </is>
       </c>
       <c r="H362" s="1" t="n">
-        <v>12.66</v>
+        <v>12.67</v>
       </c>
     </row>
     <row r="363">
@@ -12654,7 +12654,7 @@
         </is>
       </c>
       <c r="H365" s="1" t="n">
-        <v>34.54</v>
+        <v>34.5</v>
       </c>
     </row>
     <row r="366">
@@ -12687,7 +12687,7 @@
         </is>
       </c>
       <c r="H366" s="1" t="n">
-        <v>5.29</v>
+        <v>5.31</v>
       </c>
     </row>
     <row r="367">
@@ -12720,7 +12720,7 @@
         </is>
       </c>
       <c r="H367" s="1" t="n">
-        <v>253.75</v>
+        <v>254</v>
       </c>
     </row>
     <row r="368">
@@ -12753,7 +12753,7 @@
         </is>
       </c>
       <c r="H368" s="1" t="n">
-        <v>159.8</v>
+        <v>159.7</v>
       </c>
     </row>
     <row r="369">
@@ -12786,7 +12786,7 @@
         </is>
       </c>
       <c r="H369" s="1" t="n">
-        <v>19.88</v>
+        <v>19.86</v>
       </c>
     </row>
     <row r="370">
@@ -12819,7 +12819,7 @@
         </is>
       </c>
       <c r="H370" s="1" t="n">
-        <v>9.529999999999999</v>
+        <v>9.539999999999999</v>
       </c>
     </row>
     <row r="371">
@@ -12852,7 +12852,7 @@
         </is>
       </c>
       <c r="H371" s="1" t="n">
-        <v>8.48</v>
+        <v>8.58</v>
       </c>
     </row>
     <row r="372">
@@ -12905,7 +12905,7 @@
         </is>
       </c>
       <c r="D373" s="1" t="n">
-        <v>7.523352</v>
+        <v>7.436174</v>
       </c>
       <c r="F373" t="inlineStr">
         <is>
@@ -12938,7 +12938,7 @@
         </is>
       </c>
       <c r="D374" s="1" t="n">
-        <v>9.74569</v>
+        <v>9.765241</v>
       </c>
       <c r="F374" t="inlineStr">
         <is>
@@ -12951,7 +12951,7 @@
         </is>
       </c>
       <c r="H374" s="1" t="n">
-        <v>98.34999999999999</v>
+        <v>98.5</v>
       </c>
     </row>
     <row r="375">
@@ -12984,7 +12984,7 @@
         </is>
       </c>
       <c r="H375" s="1" t="n">
-        <v>80.5</v>
+        <v>80.55</v>
       </c>
     </row>
     <row r="376">
@@ -13017,7 +13017,7 @@
         </is>
       </c>
       <c r="H376" s="1" t="n">
-        <v>9.109999999999999</v>
+        <v>9.130000000000001</v>
       </c>
     </row>
     <row r="377">
@@ -13050,7 +13050,7 @@
         </is>
       </c>
       <c r="H377" s="1" t="n">
-        <v>24.12</v>
+        <v>24</v>
       </c>
     </row>
     <row r="378">
@@ -13116,7 +13116,7 @@
         </is>
       </c>
       <c r="H379" s="1" t="n">
-        <v>3.73</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="380">
@@ -13182,7 +13182,7 @@
         </is>
       </c>
       <c r="H381" s="1" t="n">
-        <v>6.13</v>
+        <v>6.12</v>
       </c>
     </row>
     <row r="382">
@@ -13215,7 +13215,7 @@
         </is>
       </c>
       <c r="H382" s="1" t="n">
-        <v>11.44</v>
+        <v>11.49</v>
       </c>
     </row>
     <row r="383">
@@ -13248,7 +13248,7 @@
         </is>
       </c>
       <c r="H383" s="1" t="n">
-        <v>1.88</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="384">
@@ -13281,7 +13281,7 @@
         </is>
       </c>
       <c r="H384" s="1" t="n">
-        <v>65.05</v>
+        <v>65.09999999999999</v>
       </c>
     </row>
     <row r="385">
@@ -13314,7 +13314,7 @@
         </is>
       </c>
       <c r="H385" s="1" t="n">
-        <v>117.2</v>
+        <v>116.7</v>
       </c>
     </row>
     <row r="386">
@@ -13334,7 +13334,7 @@
         </is>
       </c>
       <c r="D386" s="1" t="n">
-        <v>2.726937</v>
+        <v>2.708853</v>
       </c>
       <c r="F386" t="inlineStr">
         <is>
@@ -13347,7 +13347,7 @@
         </is>
       </c>
       <c r="H386" s="1" t="n">
-        <v>4.31</v>
+        <v>4.32</v>
       </c>
     </row>
     <row r="387">
@@ -13380,7 +13380,7 @@
         </is>
       </c>
       <c r="H387" s="1" t="n">
-        <v>21.46</v>
+        <v>21.48</v>
       </c>
     </row>
     <row r="388">
@@ -13413,7 +13413,7 @@
         </is>
       </c>
       <c r="H388" s="1" t="n">
-        <v>16</v>
+        <v>16.06</v>
       </c>
     </row>
     <row r="389">
@@ -13446,7 +13446,7 @@
         </is>
       </c>
       <c r="H389" s="1" t="n">
-        <v>56.05</v>
+        <v>56.4</v>
       </c>
     </row>
     <row r="390">
@@ -13479,7 +13479,7 @@
         </is>
       </c>
       <c r="H390" s="1" t="n">
-        <v>8.98</v>
+        <v>8.92</v>
       </c>
     </row>
     <row r="391">
@@ -13512,7 +13512,7 @@
         </is>
       </c>
       <c r="H391" s="1" t="n">
-        <v>24.9</v>
+        <v>24.62</v>
       </c>
     </row>
     <row r="392">
@@ -13532,7 +13532,7 @@
         </is>
       </c>
       <c r="D392" s="1" t="n">
-        <v>0</v>
+        <v>5.641653</v>
       </c>
       <c r="F392" t="inlineStr">
         <is>
@@ -13545,7 +13545,7 @@
         </is>
       </c>
       <c r="H392" s="1" t="n">
-        <v>67.15000000000001</v>
+        <v>66.05</v>
       </c>
     </row>
     <row r="393">
@@ -13578,7 +13578,7 @@
         </is>
       </c>
       <c r="H393" s="1" t="n">
-        <v>13.61</v>
+        <v>13.65</v>
       </c>
     </row>
     <row r="394">
@@ -13611,7 +13611,7 @@
         </is>
       </c>
       <c r="H394" s="1" t="n">
-        <v>289</v>
+        <v>288.5</v>
       </c>
     </row>
     <row r="395">
@@ -13644,7 +13644,7 @@
         </is>
       </c>
       <c r="H395" s="1" t="n">
-        <v>30.9</v>
+        <v>30.82</v>
       </c>
     </row>
     <row r="396">
@@ -13677,7 +13677,7 @@
         </is>
       </c>
       <c r="H396" s="1" t="n">
-        <v>6.87</v>
+        <v>7.08</v>
       </c>
     </row>
     <row r="397">
@@ -13710,7 +13710,7 @@
         </is>
       </c>
       <c r="H397" s="1" t="n">
-        <v>34.92</v>
+        <v>34.18</v>
       </c>
     </row>
     <row r="398">
@@ -13743,7 +13743,7 @@
         </is>
       </c>
       <c r="H398" s="1" t="n">
-        <v>5.7</v>
+        <v>5.78</v>
       </c>
     </row>
     <row r="399">
@@ -13776,7 +13776,7 @@
         </is>
       </c>
       <c r="H399" s="1" t="n">
-        <v>34.04</v>
+        <v>34.84</v>
       </c>
     </row>
     <row r="400">
@@ -13842,7 +13842,7 @@
         </is>
       </c>
       <c r="H401" s="1" t="n">
-        <v>6.49</v>
+        <v>6.51</v>
       </c>
     </row>
     <row r="402">
@@ -13875,7 +13875,7 @@
         </is>
       </c>
       <c r="H402" s="1" t="n">
-        <v>6.93</v>
+        <v>6.95</v>
       </c>
     </row>
     <row r="403">
@@ -13908,7 +13908,7 @@
         </is>
       </c>
       <c r="H403" s="1" t="n">
-        <v>2.44</v>
+        <v>2.46</v>
       </c>
     </row>
     <row r="404">
@@ -13941,7 +13941,7 @@
         </is>
       </c>
       <c r="H404" s="1" t="n">
-        <v>2.65</v>
+        <v>2.64</v>
       </c>
     </row>
     <row r="405">
@@ -13974,7 +13974,7 @@
         </is>
       </c>
       <c r="H405" s="1" t="n">
-        <v>23.6</v>
+        <v>23.78</v>
       </c>
     </row>
     <row r="406">
@@ -14007,7 +14007,7 @@
         </is>
       </c>
       <c r="H406" s="1" t="n">
-        <v>18.85</v>
+        <v>18.41</v>
       </c>
     </row>
     <row r="407">
@@ -14073,7 +14073,7 @@
         </is>
       </c>
       <c r="H408" s="1" t="n">
-        <v>7.01</v>
+        <v>7</v>
       </c>
     </row>
     <row r="409">
@@ -14106,7 +14106,7 @@
         </is>
       </c>
       <c r="H409" s="1" t="n">
-        <v>12.06</v>
+        <v>12.02</v>
       </c>
     </row>
     <row r="410">
@@ -14139,7 +14139,7 @@
         </is>
       </c>
       <c r="H410" s="1" t="n">
-        <v>59.8</v>
+        <v>59.7</v>
       </c>
     </row>
     <row r="411">
@@ -14172,7 +14172,7 @@
         </is>
       </c>
       <c r="H411" s="1" t="n">
-        <v>33.6</v>
+        <v>33.78</v>
       </c>
     </row>
     <row r="412">
@@ -14205,7 +14205,7 @@
         </is>
       </c>
       <c r="H412" s="1" t="n">
-        <v>16.62</v>
+        <v>16.49</v>
       </c>
     </row>
     <row r="413">
@@ -14271,7 +14271,7 @@
         </is>
       </c>
       <c r="H414" s="1" t="n">
-        <v>8.880000000000001</v>
+        <v>8.85</v>
       </c>
     </row>
     <row r="415">
@@ -14304,7 +14304,7 @@
         </is>
       </c>
       <c r="H415" s="1" t="n">
-        <v>9.23</v>
+        <v>9.199999999999999</v>
       </c>
     </row>
     <row r="416">
@@ -14337,7 +14337,7 @@
         </is>
       </c>
       <c r="H416" s="1" t="n">
-        <v>46.28</v>
+        <v>46.36</v>
       </c>
     </row>
     <row r="417">
@@ -14370,7 +14370,7 @@
         </is>
       </c>
       <c r="H417" s="1" t="n">
-        <v>3.67</v>
+        <v>3.68</v>
       </c>
     </row>
     <row r="418">
@@ -14403,7 +14403,7 @@
         </is>
       </c>
       <c r="H418" s="1" t="n">
-        <v>9.029999999999999</v>
+        <v>8.949999999999999</v>
       </c>
     </row>
     <row r="419">
@@ -14436,7 +14436,7 @@
         </is>
       </c>
       <c r="H419" s="1" t="n">
-        <v>11.41</v>
+        <v>11.43</v>
       </c>
     </row>
     <row r="420">
@@ -14469,7 +14469,7 @@
         </is>
       </c>
       <c r="H420" s="1" t="n">
-        <v>9.460000000000001</v>
+        <v>9.470000000000001</v>
       </c>
     </row>
     <row r="421">
@@ -14502,7 +14502,7 @@
         </is>
       </c>
       <c r="H421" s="1" t="n">
-        <v>47.12</v>
+        <v>46.7</v>
       </c>
     </row>
     <row r="422">
@@ -14568,7 +14568,7 @@
         </is>
       </c>
       <c r="H423" s="1" t="n">
-        <v>14.52</v>
+        <v>14.5</v>
       </c>
     </row>
     <row r="424">
@@ -14601,7 +14601,7 @@
         </is>
       </c>
       <c r="H424" s="1" t="n">
-        <v>27.14</v>
+        <v>27.16</v>
       </c>
     </row>
     <row r="425">
@@ -14667,7 +14667,7 @@
         </is>
       </c>
       <c r="H426" s="1" t="n">
-        <v>4.26</v>
+        <v>4.25</v>
       </c>
     </row>
     <row r="427">
@@ -14700,7 +14700,7 @@
         </is>
       </c>
       <c r="H427" s="1" t="n">
-        <v>11.42</v>
+        <v>11.44</v>
       </c>
     </row>
     <row r="428">
@@ -14766,7 +14766,7 @@
         </is>
       </c>
       <c r="H429" s="1" t="n">
-        <v>1.43</v>
+        <v>1.44</v>
       </c>
     </row>
     <row r="430">
@@ -14799,7 +14799,7 @@
         </is>
       </c>
       <c r="H430" s="1" t="n">
-        <v>48.12</v>
+        <v>48.34</v>
       </c>
     </row>
     <row r="431">
@@ -14832,7 +14832,7 @@
         </is>
       </c>
       <c r="H431" s="1" t="n">
-        <v>42.26</v>
+        <v>42</v>
       </c>
     </row>
     <row r="432">
@@ -14865,7 +14865,7 @@
         </is>
       </c>
       <c r="H432" s="1" t="n">
-        <v>84.09999999999999</v>
+        <v>84.45</v>
       </c>
     </row>
     <row r="433">
@@ -14898,7 +14898,7 @@
         </is>
       </c>
       <c r="H433" s="1" t="n">
-        <v>113.3</v>
+        <v>115.3</v>
       </c>
     </row>
     <row r="434">
@@ -14931,7 +14931,7 @@
         </is>
       </c>
       <c r="H434" s="1" t="n">
-        <v>5.99</v>
+        <v>6.03</v>
       </c>
     </row>
     <row r="435">
@@ -14964,7 +14964,7 @@
         </is>
       </c>
       <c r="H435" s="1" t="n">
-        <v>132.4</v>
+        <v>132.2</v>
       </c>
     </row>
     <row r="436">
@@ -14997,7 +14997,7 @@
         </is>
       </c>
       <c r="H436" s="1" t="n">
-        <v>24.52</v>
+        <v>24.58</v>
       </c>
     </row>
     <row r="437">
@@ -15063,7 +15063,7 @@
         </is>
       </c>
       <c r="H438" s="1" t="n">
-        <v>163.2</v>
+        <v>164.2</v>
       </c>
     </row>
     <row r="439">
@@ -15096,7 +15096,7 @@
         </is>
       </c>
       <c r="H439" s="1" t="n">
-        <v>38.3</v>
+        <v>38.52</v>
       </c>
     </row>
     <row r="440">
@@ -15195,7 +15195,7 @@
         </is>
       </c>
       <c r="H442" s="1" t="n">
-        <v>10.89</v>
+        <v>10.9</v>
       </c>
     </row>
     <row r="443">
@@ -15228,7 +15228,7 @@
         </is>
       </c>
       <c r="H443" s="1" t="n">
-        <v>82.8</v>
+        <v>82.5</v>
       </c>
     </row>
     <row r="444">
@@ -15261,7 +15261,7 @@
         </is>
       </c>
       <c r="H444" s="1" t="n">
-        <v>9.41</v>
+        <v>9.58</v>
       </c>
     </row>
     <row r="445">
@@ -15294,7 +15294,7 @@
         </is>
       </c>
       <c r="H445" s="1" t="n">
-        <v>1.07</v>
+        <v>1.06</v>
       </c>
     </row>
     <row r="446">
@@ -15327,7 +15327,7 @@
         </is>
       </c>
       <c r="H446" s="1" t="n">
-        <v>26.44</v>
+        <v>26.46</v>
       </c>
     </row>
     <row r="447">
@@ -15360,7 +15360,7 @@
         </is>
       </c>
       <c r="H447" s="1" t="n">
-        <v>10.93</v>
+        <v>10.92</v>
       </c>
     </row>
     <row r="448">
@@ -15393,7 +15393,7 @@
         </is>
       </c>
       <c r="H448" s="1" t="n">
-        <v>14.45</v>
+        <v>14.47</v>
       </c>
     </row>
     <row r="449">
@@ -15426,7 +15426,7 @@
         </is>
       </c>
       <c r="H449" s="1" t="n">
-        <v>11.63</v>
+        <v>11.59</v>
       </c>
     </row>
     <row r="450">
@@ -15492,7 +15492,7 @@
         </is>
       </c>
       <c r="H451" s="1" t="n">
-        <v>3.76</v>
+        <v>3.77</v>
       </c>
     </row>
     <row r="452">
@@ -15525,7 +15525,7 @@
         </is>
       </c>
       <c r="H452" s="1" t="n">
-        <v>7.58</v>
+        <v>7.57</v>
       </c>
     </row>
     <row r="453">
@@ -15558,7 +15558,7 @@
         </is>
       </c>
       <c r="H453" s="1" t="n">
-        <v>46.42</v>
+        <v>46.18</v>
       </c>
     </row>
     <row r="454">
@@ -15591,7 +15591,7 @@
         </is>
       </c>
       <c r="H454" s="1" t="n">
-        <v>7.16</v>
+        <v>7.18</v>
       </c>
     </row>
     <row r="455">
@@ -15624,7 +15624,7 @@
         </is>
       </c>
       <c r="H455" s="1" t="n">
-        <v>10.9</v>
+        <v>10.91</v>
       </c>
     </row>
     <row r="456">
@@ -15657,7 +15657,7 @@
         </is>
       </c>
       <c r="H456" s="1" t="n">
-        <v>19.75</v>
+        <v>19.78</v>
       </c>
     </row>
     <row r="457">
@@ -15723,7 +15723,7 @@
         </is>
       </c>
       <c r="H458" s="1" t="n">
-        <v>1748</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="459">
@@ -15822,7 +15822,7 @@
         </is>
       </c>
       <c r="H461" s="1" t="n">
-        <v>128.3</v>
+        <v>129</v>
       </c>
     </row>
     <row r="462">
@@ -15855,7 +15855,7 @@
         </is>
       </c>
       <c r="H462" s="1" t="n">
-        <v>28.86</v>
+        <v>28.92</v>
       </c>
     </row>
     <row r="463">
@@ -15888,7 +15888,7 @@
         </is>
       </c>
       <c r="H463" s="1" t="n">
-        <v>40.66</v>
+        <v>41.14</v>
       </c>
     </row>
     <row r="464">
@@ -15921,7 +15921,7 @@
         </is>
       </c>
       <c r="H464" s="1" t="n">
-        <v>12.55</v>
+        <v>12.56</v>
       </c>
     </row>
     <row r="465">
@@ -15954,7 +15954,7 @@
         </is>
       </c>
       <c r="H465" s="1" t="n">
-        <v>6.04</v>
+        <v>6.02</v>
       </c>
     </row>
     <row r="466">
@@ -15987,7 +15987,7 @@
         </is>
       </c>
       <c r="H466" s="1" t="n">
-        <v>13.22</v>
+        <v>13.19</v>
       </c>
     </row>
     <row r="467">
@@ -16020,7 +16020,7 @@
         </is>
       </c>
       <c r="H467" s="1" t="n">
-        <v>277.75</v>
+        <v>274</v>
       </c>
     </row>
     <row r="468">
@@ -16053,7 +16053,7 @@
         </is>
       </c>
       <c r="H468" s="1" t="n">
-        <v>95.59999999999999</v>
+        <v>95.40000000000001</v>
       </c>
     </row>
     <row r="469">
@@ -16086,7 +16086,7 @@
         </is>
       </c>
       <c r="H469" s="1" t="n">
-        <v>26.58</v>
+        <v>26.54</v>
       </c>
     </row>
     <row r="470">
@@ -16119,7 +16119,7 @@
         </is>
       </c>
       <c r="H470" s="1" t="n">
-        <v>19.86</v>
+        <v>19.71</v>
       </c>
     </row>
     <row r="471">
@@ -16152,7 +16152,7 @@
         </is>
       </c>
       <c r="H471" s="1" t="n">
-        <v>2.82</v>
+        <v>2.81</v>
       </c>
     </row>
     <row r="472">
@@ -16185,7 +16185,7 @@
         </is>
       </c>
       <c r="H472" s="1" t="n">
-        <v>182.4</v>
+        <v>182.9</v>
       </c>
     </row>
     <row r="473">
@@ -16218,7 +16218,7 @@
         </is>
       </c>
       <c r="H473" s="1" t="n">
-        <v>18.06</v>
+        <v>18.11</v>
       </c>
     </row>
     <row r="474">
@@ -16251,7 +16251,7 @@
         </is>
       </c>
       <c r="H474" s="1" t="n">
-        <v>9.199999999999999</v>
+        <v>9.34</v>
       </c>
     </row>
     <row r="475">
@@ -16284,7 +16284,7 @@
         </is>
       </c>
       <c r="H475" s="1" t="n">
-        <v>3.21</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="476">
@@ -16317,7 +16317,7 @@
         </is>
       </c>
       <c r="H476" s="1" t="n">
-        <v>1.72</v>
+        <v>1.74</v>
       </c>
     </row>
     <row r="477">
@@ -16350,7 +16350,7 @@
         </is>
       </c>
       <c r="H477" s="1" t="n">
-        <v>80.8</v>
+        <v>81.05</v>
       </c>
     </row>
     <row r="478">
@@ -16383,7 +16383,7 @@
         </is>
       </c>
       <c r="H478" s="1" t="n">
-        <v>7.41</v>
+        <v>7.42</v>
       </c>
     </row>
     <row r="479">
@@ -16449,7 +16449,7 @@
         </is>
       </c>
       <c r="H480" s="1" t="n">
-        <v>24.8</v>
+        <v>24.88</v>
       </c>
     </row>
     <row r="481">
@@ -16482,7 +16482,7 @@
         </is>
       </c>
       <c r="H481" s="1" t="n">
-        <v>2.49</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="482">
@@ -16515,7 +16515,7 @@
         </is>
       </c>
       <c r="H482" s="1" t="n">
-        <v>8.390000000000001</v>
+        <v>8.369999999999999</v>
       </c>
     </row>
     <row r="483">
@@ -16548,7 +16548,7 @@
         </is>
       </c>
       <c r="H483" s="1" t="n">
-        <v>20.24</v>
+        <v>20.22</v>
       </c>
     </row>
     <row r="484">
@@ -16581,7 +16581,7 @@
         </is>
       </c>
       <c r="H484" s="1" t="n">
-        <v>36.9</v>
+        <v>36.78</v>
       </c>
     </row>
     <row r="485">
@@ -16614,7 +16614,7 @@
         </is>
       </c>
       <c r="H485" s="1" t="n">
-        <v>92.84999999999999</v>
+        <v>94.2</v>
       </c>
     </row>
     <row r="486">
@@ -16647,7 +16647,7 @@
         </is>
       </c>
       <c r="H486" s="1" t="n">
-        <v>29.3</v>
+        <v>29.28</v>
       </c>
     </row>
     <row r="487">
@@ -16680,7 +16680,7 @@
         </is>
       </c>
       <c r="H487" s="1" t="n">
-        <v>3.75</v>
+        <v>3.74</v>
       </c>
     </row>
     <row r="488">
@@ -16713,7 +16713,7 @@
         </is>
       </c>
       <c r="H488" s="1" t="n">
-        <v>30.66</v>
+        <v>30.68</v>
       </c>
     </row>
     <row r="489">
@@ -16746,7 +16746,7 @@
         </is>
       </c>
       <c r="H489" s="1" t="n">
-        <v>11.35</v>
+        <v>11.36</v>
       </c>
     </row>
     <row r="490">
@@ -16779,7 +16779,7 @@
         </is>
       </c>
       <c r="H490" s="1" t="n">
-        <v>14.52</v>
+        <v>14.49</v>
       </c>
     </row>
     <row r="491">
@@ -16812,7 +16812,7 @@
         </is>
       </c>
       <c r="H491" s="1" t="n">
-        <v>10.08</v>
+        <v>10.07</v>
       </c>
     </row>
     <row r="492">
@@ -16845,7 +16845,7 @@
         </is>
       </c>
       <c r="H492" s="1" t="n">
-        <v>11.05</v>
+        <v>11.11</v>
       </c>
     </row>
     <row r="493">
@@ -16878,7 +16878,7 @@
         </is>
       </c>
       <c r="H493" s="1" t="n">
-        <v>1.92</v>
+        <v>1.91</v>
       </c>
     </row>
     <row r="494">
@@ -16911,7 +16911,7 @@
         </is>
       </c>
       <c r="H494" s="1" t="n">
-        <v>2.9</v>
+        <v>2.91</v>
       </c>
     </row>
     <row r="495">
@@ -16977,7 +16977,7 @@
         </is>
       </c>
       <c r="H496" s="1" t="n">
-        <v>1.97</v>
+        <v>1.96</v>
       </c>
     </row>
     <row r="497">
@@ -17010,7 +17010,7 @@
         </is>
       </c>
       <c r="H497" s="1" t="n">
-        <v>5.9</v>
+        <v>5.94</v>
       </c>
     </row>
     <row r="498">
@@ -17043,7 +17043,7 @@
         </is>
       </c>
       <c r="H498" s="1" t="n">
-        <v>11.84</v>
+        <v>11.83</v>
       </c>
     </row>
     <row r="499">
@@ -17109,7 +17109,7 @@
         </is>
       </c>
       <c r="H500" s="1" t="n">
-        <v>7.64</v>
+        <v>7.69</v>
       </c>
     </row>
     <row r="501">
@@ -17175,7 +17175,7 @@
         </is>
       </c>
       <c r="H502" s="1" t="n">
-        <v>44.3</v>
+        <v>44.2</v>
       </c>
     </row>
     <row r="503">
@@ -17208,7 +17208,7 @@
         </is>
       </c>
       <c r="H503" s="1" t="n">
-        <v>10.6</v>
+        <v>10.61</v>
       </c>
     </row>
     <row r="504">
@@ -17241,7 +17241,7 @@
         </is>
       </c>
       <c r="H504" s="1" t="n">
-        <v>13.19</v>
+        <v>13.22</v>
       </c>
     </row>
     <row r="505">
@@ -17274,7 +17274,7 @@
         </is>
       </c>
       <c r="H505" s="1" t="n">
-        <v>24.96</v>
+        <v>24.94</v>
       </c>
     </row>
     <row r="506">
@@ -17307,7 +17307,7 @@
         </is>
       </c>
       <c r="H506" s="1" t="n">
-        <v>20.92</v>
+        <v>20.96</v>
       </c>
     </row>
     <row r="507">
@@ -17373,7 +17373,7 @@
         </is>
       </c>
       <c r="H508" s="1" t="n">
-        <v>2.26</v>
+        <v>2.23</v>
       </c>
     </row>
     <row r="509">
@@ -17406,7 +17406,7 @@
         </is>
       </c>
       <c r="H509" s="1" t="n">
-        <v>37.46</v>
+        <v>37.38</v>
       </c>
     </row>
     <row r="510">
@@ -17439,7 +17439,7 @@
         </is>
       </c>
       <c r="H510" s="1" t="n">
-        <v>16.95</v>
+        <v>16.96</v>
       </c>
     </row>
     <row r="511">
@@ -17505,7 +17505,7 @@
         </is>
       </c>
       <c r="H512" s="1" t="n">
-        <v>27.74</v>
+        <v>26.94</v>
       </c>
     </row>
     <row r="513">
@@ -17538,7 +17538,7 @@
         </is>
       </c>
       <c r="H513" s="1" t="n">
-        <v>34.84</v>
+        <v>34.88</v>
       </c>
     </row>
     <row r="514">
@@ -17604,7 +17604,7 @@
         </is>
       </c>
       <c r="H515" s="1" t="n">
-        <v>22.16</v>
+        <v>22.22</v>
       </c>
     </row>
     <row r="516">
@@ -17637,7 +17637,7 @@
         </is>
       </c>
       <c r="H516" s="1" t="n">
-        <v>1.73</v>
+        <v>1.72</v>
       </c>
     </row>
     <row r="517">
@@ -17657,7 +17657,7 @@
         </is>
       </c>
       <c r="D517" s="1" t="n">
-        <v>2.089405</v>
+        <v>2.083648</v>
       </c>
       <c r="F517" t="inlineStr">
         <is>
@@ -17703,7 +17703,7 @@
         </is>
       </c>
       <c r="H518" s="1" t="n">
-        <v>10.5</v>
+        <v>10.55</v>
       </c>
     </row>
     <row r="519">
@@ -17769,7 +17769,7 @@
         </is>
       </c>
       <c r="H520" s="1" t="n">
-        <v>84.09999999999999</v>
+        <v>84.5</v>
       </c>
     </row>
     <row r="521">
@@ -17802,7 +17802,7 @@
         </is>
       </c>
       <c r="H521" s="1" t="n">
-        <v>8.960000000000001</v>
+        <v>8.93</v>
       </c>
     </row>
     <row r="522">
@@ -17835,7 +17835,7 @@
         </is>
       </c>
       <c r="H522" s="1" t="n">
-        <v>2.9</v>
+        <v>2.88</v>
       </c>
     </row>
     <row r="523">
@@ -17868,7 +17868,7 @@
         </is>
       </c>
       <c r="H523" s="1" t="n">
-        <v>15.49</v>
+        <v>15.46</v>
       </c>
     </row>
     <row r="524">
@@ -17892,16 +17892,16 @@
       </c>
       <c r="F524" t="inlineStr">
         <is>
-          <t>IHLGM</t>
+          <t>RTALB</t>
         </is>
       </c>
       <c r="G524" t="inlineStr">
         <is>
-          <t>İHLAS GAYRİMENKUL PROJE GELİŞTİRME VE TİCARET A.Ş.</t>
+          <t>RTA LABORATUVARLARI BİYOLOJİK ÜRÜNLER İLAÇ VE MAKİNE SANAYİ TİCARET A.Ş.</t>
         </is>
       </c>
       <c r="H524" s="1" t="n">
-        <v>1.7</v>
+        <v>3.33</v>
       </c>
     </row>
     <row r="525">
@@ -17925,16 +17925,16 @@
       </c>
       <c r="F525" t="inlineStr">
         <is>
-          <t>RTALB</t>
+          <t>IHLGM</t>
         </is>
       </c>
       <c r="G525" t="inlineStr">
         <is>
-          <t>RTA LABORATUVARLARI BİYOLOJİK ÜRÜNLER İLAÇ VE MAKİNE SANAYİ TİCARET A.Ş.</t>
+          <t>İHLAS GAYRİMENKUL PROJE GELİŞTİRME VE TİCARET A.Ş.</t>
         </is>
       </c>
       <c r="H525" s="1" t="n">
-        <v>3.33</v>
+        <v>1.69</v>
       </c>
     </row>
     <row r="526">
@@ -18033,7 +18033,7 @@
         </is>
       </c>
       <c r="H528" s="1" t="n">
-        <v>29.86</v>
+        <v>29.9</v>
       </c>
     </row>
     <row r="529">
@@ -18099,7 +18099,7 @@
         </is>
       </c>
       <c r="H530" s="1" t="n">
-        <v>2.38</v>
+        <v>2.37</v>
       </c>
     </row>
     <row r="531">
@@ -18132,7 +18132,7 @@
         </is>
       </c>
       <c r="H531" s="1" t="n">
-        <v>77</v>
+        <v>81.3</v>
       </c>
     </row>
     <row r="532">
@@ -18165,7 +18165,7 @@
         </is>
       </c>
       <c r="H532" s="1" t="n">
-        <v>9.369999999999999</v>
+        <v>9.359999999999999</v>
       </c>
     </row>
     <row r="533">
@@ -18231,7 +18231,7 @@
         </is>
       </c>
       <c r="H534" s="1" t="n">
-        <v>3.13</v>
+        <v>3.15</v>
       </c>
     </row>
     <row r="535">
@@ -18264,7 +18264,7 @@
         </is>
       </c>
       <c r="H535" s="1" t="n">
-        <v>20.64</v>
+        <v>20.66</v>
       </c>
     </row>
     <row r="536">
@@ -18330,7 +18330,7 @@
         </is>
       </c>
       <c r="H537" s="1" t="n">
-        <v>6.38</v>
+        <v>6.35</v>
       </c>
     </row>
     <row r="538">
@@ -18363,7 +18363,7 @@
         </is>
       </c>
       <c r="H538" s="1" t="n">
-        <v>7.88</v>
+        <v>7.89</v>
       </c>
     </row>
     <row r="539">
@@ -18429,7 +18429,7 @@
         </is>
       </c>
       <c r="H540" s="1" t="n">
-        <v>12.79</v>
+        <v>12.67</v>
       </c>
     </row>
     <row r="541">
@@ -18462,7 +18462,7 @@
         </is>
       </c>
       <c r="H541" s="1" t="n">
-        <v>6.06</v>
+        <v>6.07</v>
       </c>
     </row>
     <row r="542">
@@ -18495,7 +18495,7 @@
         </is>
       </c>
       <c r="H542" s="1" t="n">
-        <v>39.18</v>
+        <v>38.8</v>
       </c>
     </row>
     <row r="543">
@@ -18528,7 +18528,7 @@
         </is>
       </c>
       <c r="H543" s="1" t="n">
-        <v>8.23</v>
+        <v>8.25</v>
       </c>
     </row>
     <row r="544">
@@ -18594,7 +18594,7 @@
         </is>
       </c>
       <c r="H545" s="1" t="n">
-        <v>181.1</v>
+        <v>181.7</v>
       </c>
     </row>
     <row r="546">
@@ -18627,7 +18627,7 @@
         </is>
       </c>
       <c r="H546" s="1" t="n">
-        <v>2.38</v>
+        <v>2.39</v>
       </c>
     </row>
     <row r="547">
@@ -18693,7 +18693,7 @@
         </is>
       </c>
       <c r="H548" s="1" t="n">
-        <v>125.9</v>
+        <v>126.2</v>
       </c>
     </row>
     <row r="549">
@@ -18792,7 +18792,7 @@
         </is>
       </c>
       <c r="H551" s="1" t="n">
-        <v>28.96</v>
+        <v>28.98</v>
       </c>
     </row>
     <row r="552">
@@ -18891,7 +18891,7 @@
         </is>
       </c>
       <c r="H554" s="1" t="n">
-        <v>15.72</v>
+        <v>15.82</v>
       </c>
     </row>
     <row r="555">
@@ -18924,7 +18924,7 @@
         </is>
       </c>
       <c r="H555" s="1" t="n">
-        <v>13.14</v>
+        <v>13.15</v>
       </c>
     </row>
     <row r="556">
@@ -18957,7 +18957,7 @@
         </is>
       </c>
       <c r="H556" s="1" t="n">
-        <v>7.76</v>
+        <v>7.77</v>
       </c>
     </row>
     <row r="557">
@@ -18990,7 +18990,7 @@
         </is>
       </c>
       <c r="H557" s="1" t="n">
-        <v>1.45</v>
+        <v>1.44</v>
       </c>
     </row>
     <row r="558">
@@ -19023,7 +19023,7 @@
         </is>
       </c>
       <c r="H558" s="1" t="n">
-        <v>22.64</v>
+        <v>22.74</v>
       </c>
     </row>
     <row r="559">
@@ -19056,7 +19056,7 @@
         </is>
       </c>
       <c r="H559" s="1" t="n">
-        <v>4.58</v>
+        <v>4.6</v>
       </c>
     </row>
     <row r="560">
@@ -19089,7 +19089,7 @@
         </is>
       </c>
       <c r="H560" s="1" t="n">
-        <v>16.02</v>
+        <v>15.99</v>
       </c>
     </row>
     <row r="561">
@@ -19122,7 +19122,7 @@
         </is>
       </c>
       <c r="H561" s="1" t="n">
-        <v>10.73</v>
+        <v>10.77</v>
       </c>
     </row>
     <row r="562">
@@ -19155,7 +19155,7 @@
         </is>
       </c>
       <c r="H562" s="1" t="n">
-        <v>46.4</v>
+        <v>45.06</v>
       </c>
     </row>
     <row r="563">
@@ -19254,7 +19254,7 @@
         </is>
       </c>
       <c r="H565" s="1" t="n">
-        <v>59.25</v>
+        <v>59.05</v>
       </c>
     </row>
     <row r="566">
@@ -19287,7 +19287,7 @@
         </is>
       </c>
       <c r="H566" s="1" t="n">
-        <v>23.98</v>
+        <v>24</v>
       </c>
     </row>
     <row r="567">
@@ -19320,7 +19320,7 @@
         </is>
       </c>
       <c r="H567" s="1" t="n">
-        <v>5.48</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="568">
@@ -19353,7 +19353,7 @@
         </is>
       </c>
       <c r="H568" s="1" t="n">
-        <v>1.27</v>
+        <v>1.26</v>
       </c>
     </row>
     <row r="569">
@@ -19452,7 +19452,7 @@
         </is>
       </c>
       <c r="H571" s="1" t="n">
-        <v>23.76</v>
+        <v>23.74</v>
       </c>
     </row>
     <row r="572">
@@ -19485,7 +19485,7 @@
         </is>
       </c>
       <c r="H572" s="1" t="n">
-        <v>5.13</v>
+        <v>5.12</v>
       </c>
     </row>
     <row r="573">
@@ -19518,7 +19518,7 @@
         </is>
       </c>
       <c r="H573" s="1" t="n">
-        <v>4.87</v>
+        <v>4.86</v>
       </c>
     </row>
     <row r="574">
@@ -19551,7 +19551,7 @@
         </is>
       </c>
       <c r="H574" s="1" t="n">
-        <v>10.22</v>
+        <v>10.26</v>
       </c>
     </row>
     <row r="575">
@@ -19617,7 +19617,7 @@
         </is>
       </c>
       <c r="H576" s="1" t="n">
-        <v>4.04</v>
+        <v>4.01</v>
       </c>
     </row>
     <row r="577">
@@ -19683,7 +19683,7 @@
         </is>
       </c>
       <c r="H578" s="1" t="n">
-        <v>15.25</v>
+        <v>15.41</v>
       </c>
     </row>
     <row r="579">
@@ -19716,7 +19716,7 @@
         </is>
       </c>
       <c r="H579" s="1" t="n">
-        <v>47.12</v>
+        <v>47.18</v>
       </c>
     </row>
     <row r="580">
@@ -19749,7 +19749,7 @@
         </is>
       </c>
       <c r="H580" s="1" t="n">
-        <v>122.3</v>
+        <v>122</v>
       </c>
     </row>
     <row r="581">
@@ -19782,7 +19782,7 @@
         </is>
       </c>
       <c r="H581" s="1" t="n">
-        <v>123.1</v>
+        <v>123.6</v>
       </c>
     </row>
     <row r="582">
@@ -19815,7 +19815,7 @@
         </is>
       </c>
       <c r="H582" s="1" t="n">
-        <v>23.54</v>
+        <v>23.88</v>
       </c>
     </row>
     <row r="583">
@@ -19848,7 +19848,7 @@
         </is>
       </c>
       <c r="H583" s="1" t="n">
-        <v>2.95</v>
+        <v>2.96</v>
       </c>
     </row>
     <row r="584">
@@ -19914,7 +19914,7 @@
         </is>
       </c>
       <c r="H585" s="1" t="n">
-        <v>26.22</v>
+        <v>25.92</v>
       </c>
     </row>
     <row r="586">
@@ -19947,7 +19947,7 @@
         </is>
       </c>
       <c r="H586" s="1" t="n">
-        <v>2.34</v>
+        <v>2.35</v>
       </c>
     </row>
     <row r="587">
@@ -20046,7 +20046,7 @@
         </is>
       </c>
       <c r="H589" s="1" t="n">
-        <v>26.1</v>
+        <v>25.86</v>
       </c>
     </row>
     <row r="590">
@@ -20079,7 +20079,7 @@
         </is>
       </c>
       <c r="H590" s="1" t="n">
-        <v>12.94</v>
+        <v>12.89</v>
       </c>
     </row>
     <row r="591">
@@ -20112,7 +20112,7 @@
         </is>
       </c>
       <c r="H591" s="1" t="n">
-        <v>12.86</v>
+        <v>12.98</v>
       </c>
     </row>
     <row r="592">
@@ -20178,7 +20178,7 @@
         </is>
       </c>
       <c r="H593" s="1" t="n">
-        <v>7.72</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="594">
@@ -20211,7 +20211,7 @@
         </is>
       </c>
       <c r="H594" s="1" t="n">
-        <v>24.86</v>
+        <v>24.88</v>
       </c>
     </row>
     <row r="595">
@@ -20244,7 +20244,7 @@
         </is>
       </c>
       <c r="H595" s="1" t="n">
-        <v>2.01</v>
+        <v>2.02</v>
       </c>
     </row>
     <row r="596">
@@ -20277,7 +20277,7 @@
         </is>
       </c>
       <c r="H596" s="1" t="n">
-        <v>4.45</v>
+        <v>4.43</v>
       </c>
     </row>
     <row r="597">
@@ -20310,7 +20310,7 @@
         </is>
       </c>
       <c r="H597" s="1" t="n">
-        <v>14.95</v>
+        <v>15.18</v>
       </c>
     </row>
     <row r="598">
@@ -20343,7 +20343,7 @@
         </is>
       </c>
       <c r="H598" s="1" t="n">
-        <v>7.99</v>
+        <v>7.97</v>
       </c>
     </row>
     <row r="599">
@@ -20442,7 +20442,7 @@
         </is>
       </c>
       <c r="H601" s="1" t="n">
-        <v>2.44</v>
+        <v>2.45</v>
       </c>
     </row>
     <row r="602">
@@ -20475,7 +20475,7 @@
         </is>
       </c>
       <c r="H602" s="1" t="n">
-        <v>23.38</v>
+        <v>23.46</v>
       </c>
     </row>
     <row r="603">
@@ -20508,7 +20508,7 @@
         </is>
       </c>
       <c r="H603" s="1" t="n">
-        <v>5.53</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="604">
@@ -20541,7 +20541,7 @@
         </is>
       </c>
       <c r="H604" s="1" t="n">
-        <v>1.31</v>
+        <v>1.32</v>
       </c>
     </row>
     <row r="605">
@@ -20574,7 +20574,7 @@
         </is>
       </c>
       <c r="H605" s="1" t="n">
-        <v>14.8</v>
+        <v>14.76</v>
       </c>
     </row>
     <row r="606">
@@ -20640,7 +20640,7 @@
         </is>
       </c>
       <c r="H607" s="1" t="n">
-        <v>10.98</v>
+        <v>10.95</v>
       </c>
     </row>
     <row r="608">
@@ -20673,7 +20673,7 @@
         </is>
       </c>
       <c r="H608" s="1" t="n">
-        <v>7.6</v>
+        <v>7.56</v>
       </c>
     </row>
     <row r="609">
@@ -20706,7 +20706,7 @@
         </is>
       </c>
       <c r="H609" s="1" t="n">
-        <v>10.02</v>
+        <v>9.91</v>
       </c>
     </row>
     <row r="610">
@@ -20772,7 +20772,7 @@
         </is>
       </c>
       <c r="H611" s="1" t="n">
-        <v>5.16</v>
+        <v>5.13</v>
       </c>
     </row>
     <row r="612">
@@ -20829,16 +20829,16 @@
       </c>
       <c r="F613" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="G613" t="inlineStr">
         <is>
-          <t>Enpara Bank A.S.</t>
+          <t>Agaoglu Avrasya Gayrimenkul Yatirim Ortakligi AS</t>
         </is>
       </c>
       <c r="H613" s="1" t="n">
-        <v>61.9</v>
+        <v>14.24</v>
       </c>
     </row>
     <row r="614">
@@ -20862,16 +20862,16 @@
       </c>
       <c r="F614" t="inlineStr">
         <is>
-          <t>ORZAX</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="G614" t="inlineStr">
         <is>
-          <t>Orzaks Ilac ve Kimya Sanayi Ticaret A.S.</t>
+          <t>Luxera Gayrimenkul Yatirim Ortakligi A.S.</t>
         </is>
       </c>
       <c r="H614" s="1" t="n">
-        <v>100.3</v>
+        <v>12.77</v>
       </c>
     </row>
     <row r="615">
@@ -20895,16 +20895,16 @@
       </c>
       <c r="F615" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="G615" t="inlineStr">
         <is>
-          <t>Luxera Gayrimenkul Yatirim Ortakligi A.S.</t>
+          <t>Enpara Bank A.S.</t>
         </is>
       </c>
       <c r="H615" s="1" t="n">
-        <v>12.71</v>
+        <v>61.9</v>
       </c>
     </row>
     <row r="616">
@@ -20937,7 +20937,7 @@
         </is>
       </c>
       <c r="H616" s="1" t="n">
-        <v>87.59999999999999</v>
+        <v>89.7</v>
       </c>
     </row>
     <row r="617">
@@ -20961,16 +20961,16 @@
       </c>
       <c r="F617" t="inlineStr">
         <is>
-          <t>EKIM</t>
+          <t>ORZAX</t>
         </is>
       </c>
       <c r="G617" t="inlineStr">
         <is>
-          <t>EKİM TURİZM TİCARET VE SANAYİ A.Ş.</t>
+          <t>Orzaks Ilac ve Kimya Sanayi Ticaret A.S.</t>
         </is>
       </c>
       <c r="H617" s="1" t="n">
-        <v>21.66</v>
+        <v>100.7</v>
       </c>
     </row>
     <row r="618">
@@ -20994,16 +20994,16 @@
       </c>
       <c r="F618" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>EKIM</t>
         </is>
       </c>
       <c r="G618" t="inlineStr">
         <is>
-          <t>Agaoglu Avrasya Gayrimenkul Yatirim Ortakligi AS</t>
+          <t>EKİM TURİZM TİCARET VE SANAYİ A.Ş.</t>
         </is>
       </c>
       <c r="H618" s="1" t="n">
-        <v>14.27</v>
+        <v>21.7</v>
       </c>
     </row>
     <row r="619">
@@ -21036,7 +21036,7 @@
         </is>
       </c>
       <c r="H619" s="1" t="n">
-        <v>70.23999999999999</v>
+        <v>70.17</v>
       </c>
     </row>
     <row r="620">

</xml_diff>